<commit_message>
Planillas gratuitas: cabecera con la firma tipográfica oficial del manual de marca
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016mDSo1khrmevMxTP9De9mC
</commit_message>
<xml_diff>
--- a/gratis/archivos/gastos-hogar/Servicios_y_Gastos_del_Hogar_MixShopDigital.xlsx
+++ b/gratis/archivos/gastos-hogar/Servicios_y_Gastos_del_Hogar_MixShopDigital.xlsx
@@ -39,7 +39,7 @@
     <numFmt numFmtId="166" formatCode="#,##0;[Red]-#,##0;;@"/>
     <numFmt numFmtId="167" formatCode="0%;-0%;&quot;-&quot;"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="29">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,6 +74,12 @@
       <name val="Arial"/>
       <color rgb="00000000"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <color rgb="000B2A7A"/>
+      <sz val="13"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -207,7 +213,7 @@
       <u val="single"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="15">
     <fill>
       <patternFill/>
     </fill>
@@ -234,8 +240,44 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+        <bgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FF7A00"/>
+        <bgColor rgb="00FF7A00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFB800"/>
+        <bgColor rgb="00FFB800"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000094FB"/>
+        <bgColor rgb="000094FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FDF0DC"/>
         <bgColor rgb="00FDF0DC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002ECC40"/>
+        <bgColor rgb="002ECC40"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="008727E2"/>
+        <bgColor rgb="008727E2"/>
       </patternFill>
     </fill>
     <fill>
@@ -254,12 +296,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FAF6F1"/>
         <bgColor rgb="00FAF6F1"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FFFFFF"/>
-        <bgColor rgb="00FFFFFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -309,12 +345,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="77">
+  <cellXfs count="83">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -323,228 +360,233 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="20" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="24" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="22" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="17" fillId="13" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="1" fontId="16" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="16" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+      <protection locked="0" hidden="0"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="12" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="19" fillId="14" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="1" fontId="20" fillId="14" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="21" fillId="14" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="19" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="16" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="23" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="22" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="16" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="22" fillId="14" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="16" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="3" fontId="15" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="18" fillId="8" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="1" fontId="19" fillId="8" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="20" fillId="8" borderId="5" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="21" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="5" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="3" fontId="5" fillId="9" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-      <protection locked="0" hidden="0"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="27" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="27" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
@@ -987,6 +1029,151 @@
     </graphicFrame>
     <clientData/>
   </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1409700" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="3" name="Image 3" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId3"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1409700" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1409700" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1409700" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>1</col>
+      <colOff>57150</colOff>
+      <row>0</row>
+      <rowOff>76200</rowOff>
+    </from>
+    <ext cx="1409700" cy="285750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
 </wsDr>
 </file>
 
@@ -1299,74 +1486,91 @@
     <col hidden="1" width="13" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>MIX SHOP DIGITAL</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
+    <row r="1" ht="38" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>SERVICIOS Y GASTOS DEL HOGAR</t>
         </is>
       </c>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Tu hogar, de un vistazo</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="4" customHeight="1">
-      <c r="B3" s="5" t="n"/>
+    <row r="3" ht="5" customHeight="1">
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="8" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="9" t="n"/>
+      <c r="H3" s="9" t="n"/>
+      <c r="I3" s="9" t="n"/>
+      <c r="J3" s="10" t="n"/>
+      <c r="K3" s="10" t="n"/>
+      <c r="L3" s="11" t="n"/>
+      <c r="M3" s="11" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>El panel se arma solo con lo que anotás en SERVICIOS. No hace falta escribir nada acá, salvo elegir el período.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>+ Anotar pagos</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E5" s="14" t="inlineStr">
         <is>
           <t>Vencimientos</t>
         </is>
       </c>
-      <c r="G5" s="9" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>Ajustes</t>
         </is>
       </c>
-      <c r="I5" s="9" t="inlineStr">
+      <c r="I5" s="15" t="inlineStr">
         <is>
           <t>Ayuda</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="16" t="inlineStr">
         <is>
           <t>Período a mirar:</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="17" t="inlineStr">
         <is>
           <t>Todo el año</t>
         </is>
       </c>
-      <c r="E6" s="6">
+      <c r="E6" s="12">
         <f>"Año de control: "&amp;AnioCtl&amp;"   ·   "&amp;NombreHogar</f>
         <v/>
       </c>
@@ -1376,61 +1580,61 @@
       </c>
     </row>
     <row r="8" ht="16" customHeight="1">
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="18" t="inlineStr">
         <is>
           <t>GASTO DEL PERÍODO</t>
         </is>
       </c>
-      <c r="E8" s="13" t="inlineStr">
+      <c r="E8" s="19" t="inlineStr">
         <is>
           <t>PROMEDIO POR MES</t>
         </is>
       </c>
-      <c r="H8" s="14" t="inlineStr">
+      <c r="H8" s="20" t="inlineStr">
         <is>
           <t>VS. TU PRESUPUESTO</t>
         </is>
       </c>
-      <c r="K8" s="15" t="inlineStr">
+      <c r="K8" s="21" t="inlineStr">
         <is>
           <t>GASTO MÁS GRANDE</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="B9" s="16">
+      <c r="B9" s="22">
         <f>IF(MesN=0,C29,INDEX(C17:C28,MesN))</f>
         <v/>
       </c>
-      <c r="E9" s="17">
+      <c r="E9" s="23">
         <f>IFERROR(C29/COUNTIF(C17:C28,"&gt;0"),0)</f>
         <v/>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="24">
         <f>IF(PresMes=0,"-",IF(MesN=0,E29,INDEX(E17:E28,MesN)))</f>
         <v/>
       </c>
-      <c r="K9" s="19">
+      <c r="K9" s="25">
         <f>IF(MAX(P17:P36)&lt;=0,"-",INDEX(SERVICIOS!B8:B27,MATCH(MAX(P17:P36),P17:P36,0)))</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="15" customHeight="1">
-      <c r="B10" s="20">
+      <c r="B10" s="26">
         <f>Moneda</f>
         <v/>
       </c>
-      <c r="E10" s="21" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>meses con gastos cargados</t>
         </is>
       </c>
-      <c r="H10" s="22" t="inlineStr">
+      <c r="H10" s="28" t="inlineStr">
         <is>
           <t>positivo: te sobró · negativo: te pasaste</t>
         </is>
       </c>
-      <c r="K10" s="23" t="inlineStr">
+      <c r="K10" s="29" t="inlineStr">
         <is>
           <t>en el período</t>
         </is>
@@ -1438,61 +1642,61 @@
     </row>
     <row r="11" ht="8" customHeight="1"/>
     <row r="12" ht="24" customHeight="1">
-      <c r="B12" s="24">
+      <c r="B12" s="30">
         <f>IF(C29=0,"Cargá tus pagos en la hoja SERVICIOS para ver tu panel.",IF(AND(ISNUMBER(H9),H9&lt;0),"⚠ Te pasaste del presupuesto por "&amp;FIXED(-H9,0)&amp;" "&amp;Moneda&amp;" en este período.",IF(ISNUMBER(H9),"✔ Estás dentro de tu presupuesto.","✔ Tus gastos están cargados. Poné un presupuesto en AJUSTES para compararlo.")))</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1">
-      <c r="B13" s="25">
+      <c r="B13" s="31">
         <f>"Este mes: "&amp;VENCIMIENTOS!B8&amp;" pagado(s)  ·  "&amp;VENCIMIENTOS!D8&amp;" pendiente(s)  ·  a pagar aprox. "&amp;FIXED(VENCIMIENTOS!F8,0)&amp;" "&amp;Moneda&amp;"   (detalle en VENCIMIENTOS)"</f>
         <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="26" t="inlineStr">
+      <c r="B15" s="32" t="inlineStr">
         <is>
           <t>MES A MES</t>
         </is>
       </c>
     </row>
     <row r="16" ht="22" customHeight="1">
-      <c r="B16" s="27" t="inlineStr">
+      <c r="B16" s="33" t="inlineStr">
         <is>
           <t>Mes</t>
         </is>
       </c>
-      <c r="C16" s="27" t="inlineStr">
+      <c r="C16" s="33" t="inlineStr">
         <is>
           <t>Gasto</t>
         </is>
       </c>
-      <c r="D16" s="27" t="inlineStr">
+      <c r="D16" s="33" t="inlineStr">
         <is>
           <t>Presupuesto</t>
         </is>
       </c>
-      <c r="E16" s="27" t="inlineStr">
+      <c r="E16" s="33" t="inlineStr">
         <is>
           <t>Diferencia</t>
         </is>
       </c>
     </row>
     <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="28" t="inlineStr">
+      <c r="B17" s="34" t="inlineStr">
         <is>
           <t>Enero</t>
         </is>
       </c>
-      <c r="C17" s="29">
+      <c r="C17" s="35">
         <f>SERVICIOS!E28</f>
         <v/>
       </c>
-      <c r="D17" s="30">
+      <c r="D17" s="36">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E17" s="31">
+      <c r="E17" s="37">
         <f>IF(OR(PresMes=0,C17=0),0,D17-C17)</f>
         <v/>
       </c>
@@ -1502,20 +1706,20 @@
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
-      <c r="B18" s="32" t="inlineStr">
+      <c r="B18" s="38" t="inlineStr">
         <is>
           <t>Febrero</t>
         </is>
       </c>
-      <c r="C18" s="33">
+      <c r="C18" s="39">
         <f>SERVICIOS!F28</f>
         <v/>
       </c>
-      <c r="D18" s="34">
+      <c r="D18" s="40">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E18" s="35">
+      <c r="E18" s="41">
         <f>IF(OR(PresMes=0,C18=0),0,D18-C18)</f>
         <v/>
       </c>
@@ -1525,20 +1729,20 @@
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
-      <c r="B19" s="28" t="inlineStr">
+      <c r="B19" s="34" t="inlineStr">
         <is>
           <t>Marzo</t>
         </is>
       </c>
-      <c r="C19" s="29">
+      <c r="C19" s="35">
         <f>SERVICIOS!G28</f>
         <v/>
       </c>
-      <c r="D19" s="30">
+      <c r="D19" s="36">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E19" s="31">
+      <c r="E19" s="37">
         <f>IF(OR(PresMes=0,C19=0),0,D19-C19)</f>
         <v/>
       </c>
@@ -1548,20 +1752,20 @@
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
-      <c r="B20" s="32" t="inlineStr">
+      <c r="B20" s="38" t="inlineStr">
         <is>
           <t>Abril</t>
         </is>
       </c>
-      <c r="C20" s="33">
+      <c r="C20" s="39">
         <f>SERVICIOS!H28</f>
         <v/>
       </c>
-      <c r="D20" s="34">
+      <c r="D20" s="40">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E20" s="35">
+      <c r="E20" s="41">
         <f>IF(OR(PresMes=0,C20=0),0,D20-C20)</f>
         <v/>
       </c>
@@ -1571,20 +1775,20 @@
       </c>
     </row>
     <row r="21" ht="18" customHeight="1">
-      <c r="B21" s="28" t="inlineStr">
+      <c r="B21" s="34" t="inlineStr">
         <is>
           <t>Mayo</t>
         </is>
       </c>
-      <c r="C21" s="29">
+      <c r="C21" s="35">
         <f>SERVICIOS!I28</f>
         <v/>
       </c>
-      <c r="D21" s="30">
+      <c r="D21" s="36">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E21" s="31">
+      <c r="E21" s="37">
         <f>IF(OR(PresMes=0,C21=0),0,D21-C21)</f>
         <v/>
       </c>
@@ -1594,20 +1798,20 @@
       </c>
     </row>
     <row r="22" ht="18" customHeight="1">
-      <c r="B22" s="32" t="inlineStr">
+      <c r="B22" s="38" t="inlineStr">
         <is>
           <t>Junio</t>
         </is>
       </c>
-      <c r="C22" s="33">
+      <c r="C22" s="39">
         <f>SERVICIOS!J28</f>
         <v/>
       </c>
-      <c r="D22" s="34">
+      <c r="D22" s="40">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E22" s="35">
+      <c r="E22" s="41">
         <f>IF(OR(PresMes=0,C22=0),0,D22-C22)</f>
         <v/>
       </c>
@@ -1617,20 +1821,20 @@
       </c>
     </row>
     <row r="23" ht="18" customHeight="1">
-      <c r="B23" s="28" t="inlineStr">
+      <c r="B23" s="34" t="inlineStr">
         <is>
           <t>Julio</t>
         </is>
       </c>
-      <c r="C23" s="29">
+      <c r="C23" s="35">
         <f>SERVICIOS!K28</f>
         <v/>
       </c>
-      <c r="D23" s="30">
+      <c r="D23" s="36">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E23" s="31">
+      <c r="E23" s="37">
         <f>IF(OR(PresMes=0,C23=0),0,D23-C23)</f>
         <v/>
       </c>
@@ -1640,20 +1844,20 @@
       </c>
     </row>
     <row r="24" ht="18" customHeight="1">
-      <c r="B24" s="32" t="inlineStr">
+      <c r="B24" s="38" t="inlineStr">
         <is>
           <t>Agosto</t>
         </is>
       </c>
-      <c r="C24" s="33">
+      <c r="C24" s="39">
         <f>SERVICIOS!L28</f>
         <v/>
       </c>
-      <c r="D24" s="34">
+      <c r="D24" s="40">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E24" s="35">
+      <c r="E24" s="41">
         <f>IF(OR(PresMes=0,C24=0),0,D24-C24)</f>
         <v/>
       </c>
@@ -1663,20 +1867,20 @@
       </c>
     </row>
     <row r="25" ht="18" customHeight="1">
-      <c r="B25" s="28" t="inlineStr">
+      <c r="B25" s="34" t="inlineStr">
         <is>
           <t>Septiembre</t>
         </is>
       </c>
-      <c r="C25" s="29">
+      <c r="C25" s="35">
         <f>SERVICIOS!M28</f>
         <v/>
       </c>
-      <c r="D25" s="30">
+      <c r="D25" s="36">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E25" s="31">
+      <c r="E25" s="37">
         <f>IF(OR(PresMes=0,C25=0),0,D25-C25)</f>
         <v/>
       </c>
@@ -1686,20 +1890,20 @@
       </c>
     </row>
     <row r="26" ht="18" customHeight="1">
-      <c r="B26" s="32" t="inlineStr">
+      <c r="B26" s="38" t="inlineStr">
         <is>
           <t>Octubre</t>
         </is>
       </c>
-      <c r="C26" s="33">
+      <c r="C26" s="39">
         <f>SERVICIOS!N28</f>
         <v/>
       </c>
-      <c r="D26" s="34">
+      <c r="D26" s="40">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E26" s="35">
+      <c r="E26" s="41">
         <f>IF(OR(PresMes=0,C26=0),0,D26-C26)</f>
         <v/>
       </c>
@@ -1709,20 +1913,20 @@
       </c>
     </row>
     <row r="27" ht="18" customHeight="1">
-      <c r="B27" s="28" t="inlineStr">
+      <c r="B27" s="34" t="inlineStr">
         <is>
           <t>Noviembre</t>
         </is>
       </c>
-      <c r="C27" s="29">
+      <c r="C27" s="35">
         <f>SERVICIOS!O28</f>
         <v/>
       </c>
-      <c r="D27" s="30">
+      <c r="D27" s="36">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E27" s="31">
+      <c r="E27" s="37">
         <f>IF(OR(PresMes=0,C27=0),0,D27-C27)</f>
         <v/>
       </c>
@@ -1732,20 +1936,20 @@
       </c>
     </row>
     <row r="28" ht="18" customHeight="1">
-      <c r="B28" s="32" t="inlineStr">
+      <c r="B28" s="38" t="inlineStr">
         <is>
           <t>Diciembre</t>
         </is>
       </c>
-      <c r="C28" s="33">
+      <c r="C28" s="39">
         <f>SERVICIOS!P28</f>
         <v/>
       </c>
-      <c r="D28" s="34">
+      <c r="D28" s="40">
         <f>PresMes</f>
         <v/>
       </c>
-      <c r="E28" s="35">
+      <c r="E28" s="41">
         <f>IF(OR(PresMes=0,C28=0),0,D28-C28)</f>
         <v/>
       </c>
@@ -1755,20 +1959,20 @@
       </c>
     </row>
     <row r="29" ht="22" customHeight="1">
-      <c r="B29" s="36" t="inlineStr">
+      <c r="B29" s="42" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="C29" s="37">
+      <c r="C29" s="43">
         <f>SUM(C17:C28)</f>
         <v/>
       </c>
-      <c r="D29" s="37">
+      <c r="D29" s="43">
         <f>SUM(D17:D28)</f>
         <v/>
       </c>
-      <c r="E29" s="37">
+      <c r="E29" s="43">
         <f>SUM(E17:E28)</f>
         <v/>
       </c>
@@ -1784,7 +1988,7 @@
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="38" t="inlineStr">
+      <c r="B31" s="44" t="inlineStr">
         <is>
           <t>POR CATEGORÍA (período elegido)</t>
         </is>
@@ -1795,17 +1999,17 @@
       </c>
     </row>
     <row r="32" ht="22" customHeight="1">
-      <c r="B32" s="27" t="inlineStr">
+      <c r="B32" s="33" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="D32" s="27" t="inlineStr">
+      <c r="D32" s="33" t="inlineStr">
         <is>
           <t>Monto</t>
         </is>
       </c>
-      <c r="E32" s="27" t="inlineStr">
+      <c r="E32" s="33" t="inlineStr">
         <is>
           <t>%</t>
         </is>
@@ -1816,15 +2020,15 @@
       </c>
     </row>
     <row r="33" ht="19" customHeight="1">
-      <c r="B33" s="39">
+      <c r="B33" s="45">
         <f>IF('AJUSTES'!$B$14="","",'AJUSTES'!$B$14)</f>
         <v/>
       </c>
-      <c r="D33" s="29">
+      <c r="D33" s="35">
         <f>IF(B33="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B33,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B33,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E33" s="40">
+      <c r="E33" s="46">
         <f>IF($D$41=0,0,D33/$D$41)</f>
         <v/>
       </c>
@@ -1834,15 +2038,15 @@
       </c>
     </row>
     <row r="34" ht="19" customHeight="1">
-      <c r="B34" s="39">
+      <c r="B34" s="45">
         <f>IF('AJUSTES'!$B$15="","",'AJUSTES'!$B$15)</f>
         <v/>
       </c>
-      <c r="D34" s="29">
+      <c r="D34" s="35">
         <f>IF(B34="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B34,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B34,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E34" s="40">
+      <c r="E34" s="46">
         <f>IF($D$41=0,0,D34/$D$41)</f>
         <v/>
       </c>
@@ -1852,15 +2056,15 @@
       </c>
     </row>
     <row r="35" ht="19" customHeight="1">
-      <c r="B35" s="39">
+      <c r="B35" s="45">
         <f>IF('AJUSTES'!$B$16="","",'AJUSTES'!$B$16)</f>
         <v/>
       </c>
-      <c r="D35" s="29">
+      <c r="D35" s="35">
         <f>IF(B35="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B35,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B35,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E35" s="40">
+      <c r="E35" s="46">
         <f>IF($D$41=0,0,D35/$D$41)</f>
         <v/>
       </c>
@@ -1870,15 +2074,15 @@
       </c>
     </row>
     <row r="36" ht="19" customHeight="1">
-      <c r="B36" s="39">
+      <c r="B36" s="45">
         <f>IF('AJUSTES'!$B$17="","",'AJUSTES'!$B$17)</f>
         <v/>
       </c>
-      <c r="D36" s="29">
+      <c r="D36" s="35">
         <f>IF(B36="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B36,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B36,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E36" s="40">
+      <c r="E36" s="46">
         <f>IF($D$41=0,0,D36/$D$41)</f>
         <v/>
       </c>
@@ -1888,88 +2092,88 @@
       </c>
     </row>
     <row r="37" ht="19" customHeight="1">
-      <c r="B37" s="39">
+      <c r="B37" s="45">
         <f>IF('AJUSTES'!$B$18="","",'AJUSTES'!$B$18)</f>
         <v/>
       </c>
-      <c r="D37" s="29">
+      <c r="D37" s="35">
         <f>IF(B37="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B37,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B37,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E37" s="40">
+      <c r="E37" s="46">
         <f>IF($D$41=0,0,D37/$D$41)</f>
         <v/>
       </c>
     </row>
     <row r="38" ht="19" customHeight="1">
-      <c r="B38" s="39">
+      <c r="B38" s="45">
         <f>IF('AJUSTES'!$B$19="","",'AJUSTES'!$B$19)</f>
         <v/>
       </c>
-      <c r="D38" s="29">
+      <c r="D38" s="35">
         <f>IF(B38="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B38,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B38,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E38" s="40">
+      <c r="E38" s="46">
         <f>IF($D$41=0,0,D38/$D$41)</f>
         <v/>
       </c>
     </row>
     <row r="39" ht="19" customHeight="1">
-      <c r="B39" s="39">
+      <c r="B39" s="45">
         <f>IF('AJUSTES'!$B$20="","",'AJUSTES'!$B$20)</f>
         <v/>
       </c>
-      <c r="D39" s="29">
+      <c r="D39" s="35">
         <f>IF(B39="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B39,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B39,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E39" s="40">
+      <c r="E39" s="46">
         <f>IF($D$41=0,0,D39/$D$41)</f>
         <v/>
       </c>
     </row>
     <row r="40" ht="19" customHeight="1">
-      <c r="B40" s="39">
+      <c r="B40" s="45">
         <f>IF('AJUSTES'!$B$21="","",'AJUSTES'!$B$21)</f>
         <v/>
       </c>
-      <c r="D40" s="29">
+      <c r="D40" s="35">
         <f>IF(B40="",0,IF(MesN=0,SUMIF(SERVICIOS!$C$8:$C$27,B40,SERVICIOS!$Q$8:$Q$27),SUMIF(SERVICIOS!$C$8:$C$27,B40,INDEX(SERVICIOS!$E$8:$P$27,0,MesN))))</f>
         <v/>
       </c>
-      <c r="E40" s="40">
+      <c r="E40" s="46">
         <f>IF($D$41=0,0,D40/$D$41)</f>
         <v/>
       </c>
     </row>
     <row r="41" ht="20" customHeight="1">
-      <c r="B41" s="41" t="inlineStr">
+      <c r="B41" s="47" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D41" s="37">
+      <c r="D41" s="43">
         <f>SUM(D33:D40)</f>
         <v/>
       </c>
-      <c r="E41" s="42">
+      <c r="E41" s="48">
         <f>SUM(E33:E40)</f>
         <v/>
       </c>
     </row>
     <row r="47" ht="8" customHeight="1">
-      <c r="B47" s="43" t="n"/>
+      <c r="B47" s="49" t="n"/>
     </row>
     <row r="48" ht="16" customHeight="1">
-      <c r="B48" s="44" t="inlineStr">
+      <c r="B48" s="50" t="inlineStr">
         <is>
           <t>MIX SHOP DIGITAL  ·  Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
     </row>
     <row r="49" ht="16" customHeight="1">
-      <c r="B49" s="45" t="inlineStr">
+      <c r="B49" s="51" t="inlineStr">
         <is>
           <t>Versión gratuita  ·  Más herramientas gratuitas para tu vida diaria  →  mixshopdigital.com.py</t>
         </is>
@@ -1977,7 +2181,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="ECF5"/>
-  <mergeCells count="41">
+  <mergeCells count="40">
     <mergeCell ref="E10:G10"/>
     <mergeCell ref="B48:M48"/>
     <mergeCell ref="C6:D6"/>
@@ -2008,7 +2212,6 @@
     <mergeCell ref="B1:E1"/>
     <mergeCell ref="H10:J10"/>
     <mergeCell ref="B33:C33"/>
-    <mergeCell ref="B3:M3"/>
     <mergeCell ref="K9:M9"/>
     <mergeCell ref="B15:F15"/>
     <mergeCell ref="E8:G8"/>
@@ -2111,48 +2314,75 @@
     <col width="13" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>MIX SHOP DIGITAL</t>
-        </is>
-      </c>
-      <c r="F1" s="2" t="inlineStr">
+    <row r="1" ht="38" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="2" t="n"/>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>SERVICIOS</t>
         </is>
       </c>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+      <c r="I1" s="2" t="n"/>
+      <c r="J1" s="2" t="n"/>
+      <c r="K1" s="2" t="n"/>
+      <c r="L1" s="2" t="n"/>
+      <c r="M1" s="2" t="n"/>
+      <c r="N1" s="2" t="n"/>
+      <c r="O1" s="2" t="n"/>
+      <c r="P1" s="2" t="n"/>
+      <c r="Q1" s="2" t="n"/>
+      <c r="R1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="F2" s="5" t="inlineStr">
         <is>
           <t>Anotá lo que pagás cada mes</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="4" customHeight="1">
-      <c r="B3" s="5" t="n"/>
+    <row r="3" ht="5" customHeight="1">
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="7" t="n"/>
+      <c r="E3" s="7" t="n"/>
+      <c r="F3" s="8" t="n"/>
+      <c r="G3" s="8" t="n"/>
+      <c r="H3" s="8" t="n"/>
+      <c r="I3" s="9" t="n"/>
+      <c r="J3" s="9" t="n"/>
+      <c r="K3" s="9" t="n"/>
+      <c r="L3" s="9" t="n"/>
+      <c r="M3" s="10" t="n"/>
+      <c r="N3" s="10" t="n"/>
+      <c r="O3" s="10" t="n"/>
+      <c r="P3" s="11" t="n"/>
+      <c r="Q3" s="11" t="n"/>
+      <c r="R3" s="11" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="46" t="n"/>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="B4" s="52" t="n"/>
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Una fila por servicio o gasto fijo. Escribí cuánto pagaste en cada mes. Se pinta de naranja si sube más de 20 % respecto del mes anterior.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>←  Volver al PANEL</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Vencimientos</t>
         </is>
@@ -2160,747 +2390,747 @@
     </row>
     <row r="6" ht="6" customHeight="1"/>
     <row r="7" ht="30" customHeight="1">
-      <c r="B7" s="47" t="inlineStr">
+      <c r="B7" s="53" t="inlineStr">
         <is>
           <t>Servicio o gasto</t>
         </is>
       </c>
-      <c r="C7" s="47" t="inlineStr">
+      <c r="C7" s="53" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="D7" s="47" t="inlineStr">
+      <c r="D7" s="53" t="inlineStr">
         <is>
           <t>Vence el día</t>
         </is>
       </c>
-      <c r="E7" s="47" t="inlineStr">
+      <c r="E7" s="53" t="inlineStr">
         <is>
           <t>Ene</t>
         </is>
       </c>
-      <c r="F7" s="47" t="inlineStr">
+      <c r="F7" s="53" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="G7" s="47" t="inlineStr">
+      <c r="G7" s="53" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="H7" s="47" t="inlineStr">
+      <c r="H7" s="53" t="inlineStr">
         <is>
           <t>Abr</t>
         </is>
       </c>
-      <c r="I7" s="47" t="inlineStr">
+      <c r="I7" s="53" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="J7" s="47" t="inlineStr">
+      <c r="J7" s="53" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="K7" s="47" t="inlineStr">
+      <c r="K7" s="53" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="L7" s="47" t="inlineStr">
+      <c r="L7" s="53" t="inlineStr">
         <is>
           <t>Ago</t>
         </is>
       </c>
-      <c r="M7" s="47" t="inlineStr">
+      <c r="M7" s="53" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="N7" s="47" t="inlineStr">
+      <c r="N7" s="53" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="O7" s="47" t="inlineStr">
+      <c r="O7" s="53" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="P7" s="47" t="inlineStr">
+      <c r="P7" s="53" t="inlineStr">
         <is>
           <t>Dic</t>
         </is>
       </c>
-      <c r="Q7" s="47" t="inlineStr">
+      <c r="Q7" s="53" t="inlineStr">
         <is>
           <t>Total del año</t>
         </is>
       </c>
-      <c r="R7" s="47" t="inlineStr">
+      <c r="R7" s="53" t="inlineStr">
         <is>
           <t>Promedio por mes</t>
         </is>
       </c>
     </row>
     <row r="8" ht="19" customHeight="1">
-      <c r="B8" s="48" t="inlineStr">
+      <c r="B8" s="54" t="inlineStr">
         <is>
           <t>Agua</t>
         </is>
       </c>
-      <c r="C8" s="49" t="inlineStr">
+      <c r="C8" s="55" t="inlineStr">
         <is>
           <t>Servicios básicos</t>
         </is>
       </c>
-      <c r="D8" s="50" t="n"/>
-      <c r="E8" s="51" t="n"/>
-      <c r="F8" s="51" t="n"/>
-      <c r="G8" s="51" t="n"/>
-      <c r="H8" s="51" t="n"/>
-      <c r="I8" s="51" t="n"/>
-      <c r="J8" s="51" t="n"/>
-      <c r="K8" s="51" t="n"/>
-      <c r="L8" s="51" t="n"/>
-      <c r="M8" s="51" t="n"/>
-      <c r="N8" s="51" t="n"/>
-      <c r="O8" s="51" t="n"/>
-      <c r="P8" s="51" t="n"/>
-      <c r="Q8" s="52">
+      <c r="D8" s="56" t="n"/>
+      <c r="E8" s="57" t="n"/>
+      <c r="F8" s="57" t="n"/>
+      <c r="G8" s="57" t="n"/>
+      <c r="H8" s="57" t="n"/>
+      <c r="I8" s="57" t="n"/>
+      <c r="J8" s="57" t="n"/>
+      <c r="K8" s="57" t="n"/>
+      <c r="L8" s="57" t="n"/>
+      <c r="M8" s="57" t="n"/>
+      <c r="N8" s="57" t="n"/>
+      <c r="O8" s="57" t="n"/>
+      <c r="P8" s="57" t="n"/>
+      <c r="Q8" s="58">
         <f>IF($B8="","",SUM(E8:P8))</f>
         <v/>
       </c>
-      <c r="R8" s="53">
+      <c r="R8" s="59">
         <f>IF($B8="","",IFERROR(Q8/COUNTIF(E8:P8,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="19" customHeight="1">
-      <c r="B9" s="48" t="inlineStr">
+      <c r="B9" s="54" t="inlineStr">
         <is>
           <t>Luz</t>
         </is>
       </c>
-      <c r="C9" s="49" t="inlineStr">
+      <c r="C9" s="55" t="inlineStr">
         <is>
           <t>Servicios básicos</t>
         </is>
       </c>
-      <c r="D9" s="50" t="n"/>
-      <c r="E9" s="51" t="n"/>
-      <c r="F9" s="51" t="n"/>
-      <c r="G9" s="51" t="n"/>
-      <c r="H9" s="51" t="n"/>
-      <c r="I9" s="51" t="n"/>
-      <c r="J9" s="51" t="n"/>
-      <c r="K9" s="51" t="n"/>
-      <c r="L9" s="51" t="n"/>
-      <c r="M9" s="51" t="n"/>
-      <c r="N9" s="51" t="n"/>
-      <c r="O9" s="51" t="n"/>
-      <c r="P9" s="51" t="n"/>
-      <c r="Q9" s="52">
+      <c r="D9" s="56" t="n"/>
+      <c r="E9" s="57" t="n"/>
+      <c r="F9" s="57" t="n"/>
+      <c r="G9" s="57" t="n"/>
+      <c r="H9" s="57" t="n"/>
+      <c r="I9" s="57" t="n"/>
+      <c r="J9" s="57" t="n"/>
+      <c r="K9" s="57" t="n"/>
+      <c r="L9" s="57" t="n"/>
+      <c r="M9" s="57" t="n"/>
+      <c r="N9" s="57" t="n"/>
+      <c r="O9" s="57" t="n"/>
+      <c r="P9" s="57" t="n"/>
+      <c r="Q9" s="58">
         <f>IF($B9="","",SUM(E9:P9))</f>
         <v/>
       </c>
-      <c r="R9" s="53">
+      <c r="R9" s="59">
         <f>IF($B9="","",IFERROR(Q9/COUNTIF(E9:P9,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="19" customHeight="1">
-      <c r="B10" s="48" t="inlineStr">
+      <c r="B10" s="54" t="inlineStr">
         <is>
           <t>Gas</t>
         </is>
       </c>
-      <c r="C10" s="49" t="inlineStr">
+      <c r="C10" s="55" t="inlineStr">
         <is>
           <t>Servicios básicos</t>
         </is>
       </c>
-      <c r="D10" s="50" t="n"/>
-      <c r="E10" s="51" t="n"/>
-      <c r="F10" s="51" t="n"/>
-      <c r="G10" s="51" t="n"/>
-      <c r="H10" s="51" t="n"/>
-      <c r="I10" s="51" t="n"/>
-      <c r="J10" s="51" t="n"/>
-      <c r="K10" s="51" t="n"/>
-      <c r="L10" s="51" t="n"/>
-      <c r="M10" s="51" t="n"/>
-      <c r="N10" s="51" t="n"/>
-      <c r="O10" s="51" t="n"/>
-      <c r="P10" s="51" t="n"/>
-      <c r="Q10" s="52">
+      <c r="D10" s="56" t="n"/>
+      <c r="E10" s="57" t="n"/>
+      <c r="F10" s="57" t="n"/>
+      <c r="G10" s="57" t="n"/>
+      <c r="H10" s="57" t="n"/>
+      <c r="I10" s="57" t="n"/>
+      <c r="J10" s="57" t="n"/>
+      <c r="K10" s="57" t="n"/>
+      <c r="L10" s="57" t="n"/>
+      <c r="M10" s="57" t="n"/>
+      <c r="N10" s="57" t="n"/>
+      <c r="O10" s="57" t="n"/>
+      <c r="P10" s="57" t="n"/>
+      <c r="Q10" s="58">
         <f>IF($B10="","",SUM(E10:P10))</f>
         <v/>
       </c>
-      <c r="R10" s="53">
+      <c r="R10" s="59">
         <f>IF($B10="","",IFERROR(Q10/COUNTIF(E10:P10,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="11" ht="19" customHeight="1">
-      <c r="B11" s="48" t="inlineStr">
+      <c r="B11" s="54" t="inlineStr">
         <is>
           <t>Internet</t>
         </is>
       </c>
-      <c r="C11" s="49" t="inlineStr">
+      <c r="C11" s="55" t="inlineStr">
         <is>
           <t>Comunicaciones</t>
         </is>
       </c>
-      <c r="D11" s="50" t="n"/>
-      <c r="E11" s="51" t="n"/>
-      <c r="F11" s="51" t="n"/>
-      <c r="G11" s="51" t="n"/>
-      <c r="H11" s="51" t="n"/>
-      <c r="I11" s="51" t="n"/>
-      <c r="J11" s="51" t="n"/>
-      <c r="K11" s="51" t="n"/>
-      <c r="L11" s="51" t="n"/>
-      <c r="M11" s="51" t="n"/>
-      <c r="N11" s="51" t="n"/>
-      <c r="O11" s="51" t="n"/>
-      <c r="P11" s="51" t="n"/>
-      <c r="Q11" s="52">
+      <c r="D11" s="56" t="n"/>
+      <c r="E11" s="57" t="n"/>
+      <c r="F11" s="57" t="n"/>
+      <c r="G11" s="57" t="n"/>
+      <c r="H11" s="57" t="n"/>
+      <c r="I11" s="57" t="n"/>
+      <c r="J11" s="57" t="n"/>
+      <c r="K11" s="57" t="n"/>
+      <c r="L11" s="57" t="n"/>
+      <c r="M11" s="57" t="n"/>
+      <c r="N11" s="57" t="n"/>
+      <c r="O11" s="57" t="n"/>
+      <c r="P11" s="57" t="n"/>
+      <c r="Q11" s="58">
         <f>IF($B11="","",SUM(E11:P11))</f>
         <v/>
       </c>
-      <c r="R11" s="53">
+      <c r="R11" s="59">
         <f>IF($B11="","",IFERROR(Q11/COUNTIF(E11:P11,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="19" customHeight="1">
-      <c r="B12" s="48" t="inlineStr">
+      <c r="B12" s="54" t="inlineStr">
         <is>
           <t>Cable / TV</t>
         </is>
       </c>
-      <c r="C12" s="49" t="inlineStr">
+      <c r="C12" s="55" t="inlineStr">
         <is>
           <t>Comunicaciones</t>
         </is>
       </c>
-      <c r="D12" s="50" t="n"/>
-      <c r="E12" s="51" t="n"/>
-      <c r="F12" s="51" t="n"/>
-      <c r="G12" s="51" t="n"/>
-      <c r="H12" s="51" t="n"/>
-      <c r="I12" s="51" t="n"/>
-      <c r="J12" s="51" t="n"/>
-      <c r="K12" s="51" t="n"/>
-      <c r="L12" s="51" t="n"/>
-      <c r="M12" s="51" t="n"/>
-      <c r="N12" s="51" t="n"/>
-      <c r="O12" s="51" t="n"/>
-      <c r="P12" s="51" t="n"/>
-      <c r="Q12" s="52">
+      <c r="D12" s="56" t="n"/>
+      <c r="E12" s="57" t="n"/>
+      <c r="F12" s="57" t="n"/>
+      <c r="G12" s="57" t="n"/>
+      <c r="H12" s="57" t="n"/>
+      <c r="I12" s="57" t="n"/>
+      <c r="J12" s="57" t="n"/>
+      <c r="K12" s="57" t="n"/>
+      <c r="L12" s="57" t="n"/>
+      <c r="M12" s="57" t="n"/>
+      <c r="N12" s="57" t="n"/>
+      <c r="O12" s="57" t="n"/>
+      <c r="P12" s="57" t="n"/>
+      <c r="Q12" s="58">
         <f>IF($B12="","",SUM(E12:P12))</f>
         <v/>
       </c>
-      <c r="R12" s="53">
+      <c r="R12" s="59">
         <f>IF($B12="","",IFERROR(Q12/COUNTIF(E12:P12,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="19" customHeight="1">
-      <c r="B13" s="48" t="inlineStr">
+      <c r="B13" s="54" t="inlineStr">
         <is>
           <t>Teléfono celular</t>
         </is>
       </c>
-      <c r="C13" s="49" t="inlineStr">
+      <c r="C13" s="55" t="inlineStr">
         <is>
           <t>Comunicaciones</t>
         </is>
       </c>
-      <c r="D13" s="50" t="n"/>
-      <c r="E13" s="51" t="n"/>
-      <c r="F13" s="51" t="n"/>
-      <c r="G13" s="51" t="n"/>
-      <c r="H13" s="51" t="n"/>
-      <c r="I13" s="51" t="n"/>
-      <c r="J13" s="51" t="n"/>
-      <c r="K13" s="51" t="n"/>
-      <c r="L13" s="51" t="n"/>
-      <c r="M13" s="51" t="n"/>
-      <c r="N13" s="51" t="n"/>
-      <c r="O13" s="51" t="n"/>
-      <c r="P13" s="51" t="n"/>
-      <c r="Q13" s="52">
+      <c r="D13" s="56" t="n"/>
+      <c r="E13" s="57" t="n"/>
+      <c r="F13" s="57" t="n"/>
+      <c r="G13" s="57" t="n"/>
+      <c r="H13" s="57" t="n"/>
+      <c r="I13" s="57" t="n"/>
+      <c r="J13" s="57" t="n"/>
+      <c r="K13" s="57" t="n"/>
+      <c r="L13" s="57" t="n"/>
+      <c r="M13" s="57" t="n"/>
+      <c r="N13" s="57" t="n"/>
+      <c r="O13" s="57" t="n"/>
+      <c r="P13" s="57" t="n"/>
+      <c r="Q13" s="58">
         <f>IF($B13="","",SUM(E13:P13))</f>
         <v/>
       </c>
-      <c r="R13" s="53">
+      <c r="R13" s="59">
         <f>IF($B13="","",IFERROR(Q13/COUNTIF(E13:P13,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="19" customHeight="1">
-      <c r="B14" s="48" t="inlineStr">
+      <c r="B14" s="54" t="inlineStr">
         <is>
           <t>Alquiler o cuota de la casa</t>
         </is>
       </c>
-      <c r="C14" s="49" t="inlineStr">
+      <c r="C14" s="55" t="inlineStr">
         <is>
           <t>Vivienda</t>
         </is>
       </c>
-      <c r="D14" s="50" t="n"/>
-      <c r="E14" s="51" t="n"/>
-      <c r="F14" s="51" t="n"/>
-      <c r="G14" s="51" t="n"/>
-      <c r="H14" s="51" t="n"/>
-      <c r="I14" s="51" t="n"/>
-      <c r="J14" s="51" t="n"/>
-      <c r="K14" s="51" t="n"/>
-      <c r="L14" s="51" t="n"/>
-      <c r="M14" s="51" t="n"/>
-      <c r="N14" s="51" t="n"/>
-      <c r="O14" s="51" t="n"/>
-      <c r="P14" s="51" t="n"/>
-      <c r="Q14" s="52">
+      <c r="D14" s="56" t="n"/>
+      <c r="E14" s="57" t="n"/>
+      <c r="F14" s="57" t="n"/>
+      <c r="G14" s="57" t="n"/>
+      <c r="H14" s="57" t="n"/>
+      <c r="I14" s="57" t="n"/>
+      <c r="J14" s="57" t="n"/>
+      <c r="K14" s="57" t="n"/>
+      <c r="L14" s="57" t="n"/>
+      <c r="M14" s="57" t="n"/>
+      <c r="N14" s="57" t="n"/>
+      <c r="O14" s="57" t="n"/>
+      <c r="P14" s="57" t="n"/>
+      <c r="Q14" s="58">
         <f>IF($B14="","",SUM(E14:P14))</f>
         <v/>
       </c>
-      <c r="R14" s="53">
+      <c r="R14" s="59">
         <f>IF($B14="","",IFERROR(Q14/COUNTIF(E14:P14,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="19" customHeight="1">
-      <c r="B15" s="48" t="inlineStr">
+      <c r="B15" s="54" t="inlineStr">
         <is>
           <t>Cuotas del colegio</t>
         </is>
       </c>
-      <c r="C15" s="49" t="inlineStr">
+      <c r="C15" s="55" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
-      <c r="D15" s="50" t="n"/>
-      <c r="E15" s="51" t="n"/>
-      <c r="F15" s="51" t="n"/>
-      <c r="G15" s="51" t="n"/>
-      <c r="H15" s="51" t="n"/>
-      <c r="I15" s="51" t="n"/>
-      <c r="J15" s="51" t="n"/>
-      <c r="K15" s="51" t="n"/>
-      <c r="L15" s="51" t="n"/>
-      <c r="M15" s="51" t="n"/>
-      <c r="N15" s="51" t="n"/>
-      <c r="O15" s="51" t="n"/>
-      <c r="P15" s="51" t="n"/>
-      <c r="Q15" s="52">
+      <c r="D15" s="56" t="n"/>
+      <c r="E15" s="57" t="n"/>
+      <c r="F15" s="57" t="n"/>
+      <c r="G15" s="57" t="n"/>
+      <c r="H15" s="57" t="n"/>
+      <c r="I15" s="57" t="n"/>
+      <c r="J15" s="57" t="n"/>
+      <c r="K15" s="57" t="n"/>
+      <c r="L15" s="57" t="n"/>
+      <c r="M15" s="57" t="n"/>
+      <c r="N15" s="57" t="n"/>
+      <c r="O15" s="57" t="n"/>
+      <c r="P15" s="57" t="n"/>
+      <c r="Q15" s="58">
         <f>IF($B15="","",SUM(E15:P15))</f>
         <v/>
       </c>
-      <c r="R15" s="53">
+      <c r="R15" s="59">
         <f>IF($B15="","",IFERROR(Q15/COUNTIF(E15:P15,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="19" customHeight="1">
-      <c r="B16" s="48" t="inlineStr">
+      <c r="B16" s="54" t="inlineStr">
         <is>
           <t>Seguro médico</t>
         </is>
       </c>
-      <c r="C16" s="49" t="inlineStr">
+      <c r="C16" s="55" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
-      <c r="D16" s="50" t="n"/>
-      <c r="E16" s="51" t="n"/>
-      <c r="F16" s="51" t="n"/>
-      <c r="G16" s="51" t="n"/>
-      <c r="H16" s="51" t="n"/>
-      <c r="I16" s="51" t="n"/>
-      <c r="J16" s="51" t="n"/>
-      <c r="K16" s="51" t="n"/>
-      <c r="L16" s="51" t="n"/>
-      <c r="M16" s="51" t="n"/>
-      <c r="N16" s="51" t="n"/>
-      <c r="O16" s="51" t="n"/>
-      <c r="P16" s="51" t="n"/>
-      <c r="Q16" s="52">
+      <c r="D16" s="56" t="n"/>
+      <c r="E16" s="57" t="n"/>
+      <c r="F16" s="57" t="n"/>
+      <c r="G16" s="57" t="n"/>
+      <c r="H16" s="57" t="n"/>
+      <c r="I16" s="57" t="n"/>
+      <c r="J16" s="57" t="n"/>
+      <c r="K16" s="57" t="n"/>
+      <c r="L16" s="57" t="n"/>
+      <c r="M16" s="57" t="n"/>
+      <c r="N16" s="57" t="n"/>
+      <c r="O16" s="57" t="n"/>
+      <c r="P16" s="57" t="n"/>
+      <c r="Q16" s="58">
         <f>IF($B16="","",SUM(E16:P16))</f>
         <v/>
       </c>
-      <c r="R16" s="53">
+      <c r="R16" s="59">
         <f>IF($B16="","",IFERROR(Q16/COUNTIF(E16:P16,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="19" customHeight="1">
-      <c r="B17" s="48" t="inlineStr">
+      <c r="B17" s="54" t="inlineStr">
         <is>
           <t>Otros gastos fijos</t>
         </is>
       </c>
-      <c r="C17" s="49" t="inlineStr">
+      <c r="C17" s="55" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>
       </c>
-      <c r="D17" s="50" t="n"/>
-      <c r="E17" s="51" t="n"/>
-      <c r="F17" s="51" t="n"/>
-      <c r="G17" s="51" t="n"/>
-      <c r="H17" s="51" t="n"/>
-      <c r="I17" s="51" t="n"/>
-      <c r="J17" s="51" t="n"/>
-      <c r="K17" s="51" t="n"/>
-      <c r="L17" s="51" t="n"/>
-      <c r="M17" s="51" t="n"/>
-      <c r="N17" s="51" t="n"/>
-      <c r="O17" s="51" t="n"/>
-      <c r="P17" s="51" t="n"/>
-      <c r="Q17" s="52">
+      <c r="D17" s="56" t="n"/>
+      <c r="E17" s="57" t="n"/>
+      <c r="F17" s="57" t="n"/>
+      <c r="G17" s="57" t="n"/>
+      <c r="H17" s="57" t="n"/>
+      <c r="I17" s="57" t="n"/>
+      <c r="J17" s="57" t="n"/>
+      <c r="K17" s="57" t="n"/>
+      <c r="L17" s="57" t="n"/>
+      <c r="M17" s="57" t="n"/>
+      <c r="N17" s="57" t="n"/>
+      <c r="O17" s="57" t="n"/>
+      <c r="P17" s="57" t="n"/>
+      <c r="Q17" s="58">
         <f>IF($B17="","",SUM(E17:P17))</f>
         <v/>
       </c>
-      <c r="R17" s="53">
+      <c r="R17" s="59">
         <f>IF($B17="","",IFERROR(Q17/COUNTIF(E17:P17,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="19" customHeight="1">
-      <c r="B18" s="48" t="n"/>
-      <c r="C18" s="49" t="n"/>
-      <c r="D18" s="50" t="n"/>
-      <c r="E18" s="51" t="n"/>
-      <c r="F18" s="51" t="n"/>
-      <c r="G18" s="51" t="n"/>
-      <c r="H18" s="51" t="n"/>
-      <c r="I18" s="51" t="n"/>
-      <c r="J18" s="51" t="n"/>
-      <c r="K18" s="51" t="n"/>
-      <c r="L18" s="51" t="n"/>
-      <c r="M18" s="51" t="n"/>
-      <c r="N18" s="51" t="n"/>
-      <c r="O18" s="51" t="n"/>
-      <c r="P18" s="51" t="n"/>
-      <c r="Q18" s="52">
+      <c r="B18" s="54" t="n"/>
+      <c r="C18" s="55" t="n"/>
+      <c r="D18" s="56" t="n"/>
+      <c r="E18" s="57" t="n"/>
+      <c r="F18" s="57" t="n"/>
+      <c r="G18" s="57" t="n"/>
+      <c r="H18" s="57" t="n"/>
+      <c r="I18" s="57" t="n"/>
+      <c r="J18" s="57" t="n"/>
+      <c r="K18" s="57" t="n"/>
+      <c r="L18" s="57" t="n"/>
+      <c r="M18" s="57" t="n"/>
+      <c r="N18" s="57" t="n"/>
+      <c r="O18" s="57" t="n"/>
+      <c r="P18" s="57" t="n"/>
+      <c r="Q18" s="58">
         <f>IF($B18="","",SUM(E18:P18))</f>
         <v/>
       </c>
-      <c r="R18" s="53">
+      <c r="R18" s="59">
         <f>IF($B18="","",IFERROR(Q18/COUNTIF(E18:P18,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="19" customHeight="1">
-      <c r="B19" s="48" t="n"/>
-      <c r="C19" s="49" t="n"/>
-      <c r="D19" s="50" t="n"/>
-      <c r="E19" s="51" t="n"/>
-      <c r="F19" s="51" t="n"/>
-      <c r="G19" s="51" t="n"/>
-      <c r="H19" s="51" t="n"/>
-      <c r="I19" s="51" t="n"/>
-      <c r="J19" s="51" t="n"/>
-      <c r="K19" s="51" t="n"/>
-      <c r="L19" s="51" t="n"/>
-      <c r="M19" s="51" t="n"/>
-      <c r="N19" s="51" t="n"/>
-      <c r="O19" s="51" t="n"/>
-      <c r="P19" s="51" t="n"/>
-      <c r="Q19" s="52">
+      <c r="B19" s="54" t="n"/>
+      <c r="C19" s="55" t="n"/>
+      <c r="D19" s="56" t="n"/>
+      <c r="E19" s="57" t="n"/>
+      <c r="F19" s="57" t="n"/>
+      <c r="G19" s="57" t="n"/>
+      <c r="H19" s="57" t="n"/>
+      <c r="I19" s="57" t="n"/>
+      <c r="J19" s="57" t="n"/>
+      <c r="K19" s="57" t="n"/>
+      <c r="L19" s="57" t="n"/>
+      <c r="M19" s="57" t="n"/>
+      <c r="N19" s="57" t="n"/>
+      <c r="O19" s="57" t="n"/>
+      <c r="P19" s="57" t="n"/>
+      <c r="Q19" s="58">
         <f>IF($B19="","",SUM(E19:P19))</f>
         <v/>
       </c>
-      <c r="R19" s="53">
+      <c r="R19" s="59">
         <f>IF($B19="","",IFERROR(Q19/COUNTIF(E19:P19,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="19" customHeight="1">
-      <c r="B20" s="48" t="n"/>
-      <c r="C20" s="49" t="n"/>
-      <c r="D20" s="50" t="n"/>
-      <c r="E20" s="51" t="n"/>
-      <c r="F20" s="51" t="n"/>
-      <c r="G20" s="51" t="n"/>
-      <c r="H20" s="51" t="n"/>
-      <c r="I20" s="51" t="n"/>
-      <c r="J20" s="51" t="n"/>
-      <c r="K20" s="51" t="n"/>
-      <c r="L20" s="51" t="n"/>
-      <c r="M20" s="51" t="n"/>
-      <c r="N20" s="51" t="n"/>
-      <c r="O20" s="51" t="n"/>
-      <c r="P20" s="51" t="n"/>
-      <c r="Q20" s="52">
+      <c r="B20" s="54" t="n"/>
+      <c r="C20" s="55" t="n"/>
+      <c r="D20" s="56" t="n"/>
+      <c r="E20" s="57" t="n"/>
+      <c r="F20" s="57" t="n"/>
+      <c r="G20" s="57" t="n"/>
+      <c r="H20" s="57" t="n"/>
+      <c r="I20" s="57" t="n"/>
+      <c r="J20" s="57" t="n"/>
+      <c r="K20" s="57" t="n"/>
+      <c r="L20" s="57" t="n"/>
+      <c r="M20" s="57" t="n"/>
+      <c r="N20" s="57" t="n"/>
+      <c r="O20" s="57" t="n"/>
+      <c r="P20" s="57" t="n"/>
+      <c r="Q20" s="58">
         <f>IF($B20="","",SUM(E20:P20))</f>
         <v/>
       </c>
-      <c r="R20" s="53">
+      <c r="R20" s="59">
         <f>IF($B20="","",IFERROR(Q20/COUNTIF(E20:P20,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="19" customHeight="1">
-      <c r="B21" s="48" t="n"/>
-      <c r="C21" s="49" t="n"/>
-      <c r="D21" s="50" t="n"/>
-      <c r="E21" s="51" t="n"/>
-      <c r="F21" s="51" t="n"/>
-      <c r="G21" s="51" t="n"/>
-      <c r="H21" s="51" t="n"/>
-      <c r="I21" s="51" t="n"/>
-      <c r="J21" s="51" t="n"/>
-      <c r="K21" s="51" t="n"/>
-      <c r="L21" s="51" t="n"/>
-      <c r="M21" s="51" t="n"/>
-      <c r="N21" s="51" t="n"/>
-      <c r="O21" s="51" t="n"/>
-      <c r="P21" s="51" t="n"/>
-      <c r="Q21" s="52">
+      <c r="B21" s="54" t="n"/>
+      <c r="C21" s="55" t="n"/>
+      <c r="D21" s="56" t="n"/>
+      <c r="E21" s="57" t="n"/>
+      <c r="F21" s="57" t="n"/>
+      <c r="G21" s="57" t="n"/>
+      <c r="H21" s="57" t="n"/>
+      <c r="I21" s="57" t="n"/>
+      <c r="J21" s="57" t="n"/>
+      <c r="K21" s="57" t="n"/>
+      <c r="L21" s="57" t="n"/>
+      <c r="M21" s="57" t="n"/>
+      <c r="N21" s="57" t="n"/>
+      <c r="O21" s="57" t="n"/>
+      <c r="P21" s="57" t="n"/>
+      <c r="Q21" s="58">
         <f>IF($B21="","",SUM(E21:P21))</f>
         <v/>
       </c>
-      <c r="R21" s="53">
+      <c r="R21" s="59">
         <f>IF($B21="","",IFERROR(Q21/COUNTIF(E21:P21,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="19" customHeight="1">
-      <c r="B22" s="48" t="n"/>
-      <c r="C22" s="49" t="n"/>
-      <c r="D22" s="50" t="n"/>
-      <c r="E22" s="51" t="n"/>
-      <c r="F22" s="51" t="n"/>
-      <c r="G22" s="51" t="n"/>
-      <c r="H22" s="51" t="n"/>
-      <c r="I22" s="51" t="n"/>
-      <c r="J22" s="51" t="n"/>
-      <c r="K22" s="51" t="n"/>
-      <c r="L22" s="51" t="n"/>
-      <c r="M22" s="51" t="n"/>
-      <c r="N22" s="51" t="n"/>
-      <c r="O22" s="51" t="n"/>
-      <c r="P22" s="51" t="n"/>
-      <c r="Q22" s="52">
+      <c r="B22" s="54" t="n"/>
+      <c r="C22" s="55" t="n"/>
+      <c r="D22" s="56" t="n"/>
+      <c r="E22" s="57" t="n"/>
+      <c r="F22" s="57" t="n"/>
+      <c r="G22" s="57" t="n"/>
+      <c r="H22" s="57" t="n"/>
+      <c r="I22" s="57" t="n"/>
+      <c r="J22" s="57" t="n"/>
+      <c r="K22" s="57" t="n"/>
+      <c r="L22" s="57" t="n"/>
+      <c r="M22" s="57" t="n"/>
+      <c r="N22" s="57" t="n"/>
+      <c r="O22" s="57" t="n"/>
+      <c r="P22" s="57" t="n"/>
+      <c r="Q22" s="58">
         <f>IF($B22="","",SUM(E22:P22))</f>
         <v/>
       </c>
-      <c r="R22" s="53">
+      <c r="R22" s="59">
         <f>IF($B22="","",IFERROR(Q22/COUNTIF(E22:P22,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="B23" s="48" t="n"/>
-      <c r="C23" s="49" t="n"/>
-      <c r="D23" s="50" t="n"/>
-      <c r="E23" s="51" t="n"/>
-      <c r="F23" s="51" t="n"/>
-      <c r="G23" s="51" t="n"/>
-      <c r="H23" s="51" t="n"/>
-      <c r="I23" s="51" t="n"/>
-      <c r="J23" s="51" t="n"/>
-      <c r="K23" s="51" t="n"/>
-      <c r="L23" s="51" t="n"/>
-      <c r="M23" s="51" t="n"/>
-      <c r="N23" s="51" t="n"/>
-      <c r="O23" s="51" t="n"/>
-      <c r="P23" s="51" t="n"/>
-      <c r="Q23" s="52">
+      <c r="B23" s="54" t="n"/>
+      <c r="C23" s="55" t="n"/>
+      <c r="D23" s="56" t="n"/>
+      <c r="E23" s="57" t="n"/>
+      <c r="F23" s="57" t="n"/>
+      <c r="G23" s="57" t="n"/>
+      <c r="H23" s="57" t="n"/>
+      <c r="I23" s="57" t="n"/>
+      <c r="J23" s="57" t="n"/>
+      <c r="K23" s="57" t="n"/>
+      <c r="L23" s="57" t="n"/>
+      <c r="M23" s="57" t="n"/>
+      <c r="N23" s="57" t="n"/>
+      <c r="O23" s="57" t="n"/>
+      <c r="P23" s="57" t="n"/>
+      <c r="Q23" s="58">
         <f>IF($B23="","",SUM(E23:P23))</f>
         <v/>
       </c>
-      <c r="R23" s="53">
+      <c r="R23" s="59">
         <f>IF($B23="","",IFERROR(Q23/COUNTIF(E23:P23,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="19" customHeight="1">
-      <c r="B24" s="48" t="n"/>
-      <c r="C24" s="49" t="n"/>
-      <c r="D24" s="50" t="n"/>
-      <c r="E24" s="51" t="n"/>
-      <c r="F24" s="51" t="n"/>
-      <c r="G24" s="51" t="n"/>
-      <c r="H24" s="51" t="n"/>
-      <c r="I24" s="51" t="n"/>
-      <c r="J24" s="51" t="n"/>
-      <c r="K24" s="51" t="n"/>
-      <c r="L24" s="51" t="n"/>
-      <c r="M24" s="51" t="n"/>
-      <c r="N24" s="51" t="n"/>
-      <c r="O24" s="51" t="n"/>
-      <c r="P24" s="51" t="n"/>
-      <c r="Q24" s="52">
+      <c r="B24" s="54" t="n"/>
+      <c r="C24" s="55" t="n"/>
+      <c r="D24" s="56" t="n"/>
+      <c r="E24" s="57" t="n"/>
+      <c r="F24" s="57" t="n"/>
+      <c r="G24" s="57" t="n"/>
+      <c r="H24" s="57" t="n"/>
+      <c r="I24" s="57" t="n"/>
+      <c r="J24" s="57" t="n"/>
+      <c r="K24" s="57" t="n"/>
+      <c r="L24" s="57" t="n"/>
+      <c r="M24" s="57" t="n"/>
+      <c r="N24" s="57" t="n"/>
+      <c r="O24" s="57" t="n"/>
+      <c r="P24" s="57" t="n"/>
+      <c r="Q24" s="58">
         <f>IF($B24="","",SUM(E24:P24))</f>
         <v/>
       </c>
-      <c r="R24" s="53">
+      <c r="R24" s="59">
         <f>IF($B24="","",IFERROR(Q24/COUNTIF(E24:P24,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="19" customHeight="1">
-      <c r="B25" s="48" t="n"/>
-      <c r="C25" s="49" t="n"/>
-      <c r="D25" s="50" t="n"/>
-      <c r="E25" s="51" t="n"/>
-      <c r="F25" s="51" t="n"/>
-      <c r="G25" s="51" t="n"/>
-      <c r="H25" s="51" t="n"/>
-      <c r="I25" s="51" t="n"/>
-      <c r="J25" s="51" t="n"/>
-      <c r="K25" s="51" t="n"/>
-      <c r="L25" s="51" t="n"/>
-      <c r="M25" s="51" t="n"/>
-      <c r="N25" s="51" t="n"/>
-      <c r="O25" s="51" t="n"/>
-      <c r="P25" s="51" t="n"/>
-      <c r="Q25" s="52">
+      <c r="B25" s="54" t="n"/>
+      <c r="C25" s="55" t="n"/>
+      <c r="D25" s="56" t="n"/>
+      <c r="E25" s="57" t="n"/>
+      <c r="F25" s="57" t="n"/>
+      <c r="G25" s="57" t="n"/>
+      <c r="H25" s="57" t="n"/>
+      <c r="I25" s="57" t="n"/>
+      <c r="J25" s="57" t="n"/>
+      <c r="K25" s="57" t="n"/>
+      <c r="L25" s="57" t="n"/>
+      <c r="M25" s="57" t="n"/>
+      <c r="N25" s="57" t="n"/>
+      <c r="O25" s="57" t="n"/>
+      <c r="P25" s="57" t="n"/>
+      <c r="Q25" s="58">
         <f>IF($B25="","",SUM(E25:P25))</f>
         <v/>
       </c>
-      <c r="R25" s="53">
+      <c r="R25" s="59">
         <f>IF($B25="","",IFERROR(Q25/COUNTIF(E25:P25,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="19" customHeight="1">
-      <c r="B26" s="48" t="n"/>
-      <c r="C26" s="49" t="n"/>
-      <c r="D26" s="50" t="n"/>
-      <c r="E26" s="51" t="n"/>
-      <c r="F26" s="51" t="n"/>
-      <c r="G26" s="51" t="n"/>
-      <c r="H26" s="51" t="n"/>
-      <c r="I26" s="51" t="n"/>
-      <c r="J26" s="51" t="n"/>
-      <c r="K26" s="51" t="n"/>
-      <c r="L26" s="51" t="n"/>
-      <c r="M26" s="51" t="n"/>
-      <c r="N26" s="51" t="n"/>
-      <c r="O26" s="51" t="n"/>
-      <c r="P26" s="51" t="n"/>
-      <c r="Q26" s="52">
+      <c r="B26" s="54" t="n"/>
+      <c r="C26" s="55" t="n"/>
+      <c r="D26" s="56" t="n"/>
+      <c r="E26" s="57" t="n"/>
+      <c r="F26" s="57" t="n"/>
+      <c r="G26" s="57" t="n"/>
+      <c r="H26" s="57" t="n"/>
+      <c r="I26" s="57" t="n"/>
+      <c r="J26" s="57" t="n"/>
+      <c r="K26" s="57" t="n"/>
+      <c r="L26" s="57" t="n"/>
+      <c r="M26" s="57" t="n"/>
+      <c r="N26" s="57" t="n"/>
+      <c r="O26" s="57" t="n"/>
+      <c r="P26" s="57" t="n"/>
+      <c r="Q26" s="58">
         <f>IF($B26="","",SUM(E26:P26))</f>
         <v/>
       </c>
-      <c r="R26" s="53">
+      <c r="R26" s="59">
         <f>IF($B26="","",IFERROR(Q26/COUNTIF(E26:P26,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="19" customHeight="1">
-      <c r="B27" s="48" t="n"/>
-      <c r="C27" s="49" t="n"/>
-      <c r="D27" s="50" t="n"/>
-      <c r="E27" s="51" t="n"/>
-      <c r="F27" s="51" t="n"/>
-      <c r="G27" s="51" t="n"/>
-      <c r="H27" s="51" t="n"/>
-      <c r="I27" s="51" t="n"/>
-      <c r="J27" s="51" t="n"/>
-      <c r="K27" s="51" t="n"/>
-      <c r="L27" s="51" t="n"/>
-      <c r="M27" s="51" t="n"/>
-      <c r="N27" s="51" t="n"/>
-      <c r="O27" s="51" t="n"/>
-      <c r="P27" s="51" t="n"/>
-      <c r="Q27" s="52">
+      <c r="B27" s="54" t="n"/>
+      <c r="C27" s="55" t="n"/>
+      <c r="D27" s="56" t="n"/>
+      <c r="E27" s="57" t="n"/>
+      <c r="F27" s="57" t="n"/>
+      <c r="G27" s="57" t="n"/>
+      <c r="H27" s="57" t="n"/>
+      <c r="I27" s="57" t="n"/>
+      <c r="J27" s="57" t="n"/>
+      <c r="K27" s="57" t="n"/>
+      <c r="L27" s="57" t="n"/>
+      <c r="M27" s="57" t="n"/>
+      <c r="N27" s="57" t="n"/>
+      <c r="O27" s="57" t="n"/>
+      <c r="P27" s="57" t="n"/>
+      <c r="Q27" s="58">
         <f>IF($B27="","",SUM(E27:P27))</f>
         <v/>
       </c>
-      <c r="R27" s="53">
+      <c r="R27" s="59">
         <f>IF($B27="","",IFERROR(Q27/COUNTIF(E27:P27,"&gt;0"),0))</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="24" customHeight="1">
-      <c r="B28" s="54" t="inlineStr">
+      <c r="B28" s="60" t="inlineStr">
         <is>
           <t>TOTAL DEL MES</t>
         </is>
       </c>
-      <c r="E28" s="37">
+      <c r="E28" s="43">
         <f>SUM(E8:E27)</f>
         <v/>
       </c>
-      <c r="F28" s="37">
+      <c r="F28" s="43">
         <f>SUM(F8:F27)</f>
         <v/>
       </c>
-      <c r="G28" s="37">
+      <c r="G28" s="43">
         <f>SUM(G8:G27)</f>
         <v/>
       </c>
-      <c r="H28" s="37">
+      <c r="H28" s="43">
         <f>SUM(H8:H27)</f>
         <v/>
       </c>
-      <c r="I28" s="37">
+      <c r="I28" s="43">
         <f>SUM(I8:I27)</f>
         <v/>
       </c>
-      <c r="J28" s="37">
+      <c r="J28" s="43">
         <f>SUM(J8:J27)</f>
         <v/>
       </c>
-      <c r="K28" s="37">
+      <c r="K28" s="43">
         <f>SUM(K8:K27)</f>
         <v/>
       </c>
-      <c r="L28" s="37">
+      <c r="L28" s="43">
         <f>SUM(L8:L27)</f>
         <v/>
       </c>
-      <c r="M28" s="37">
+      <c r="M28" s="43">
         <f>SUM(M8:M27)</f>
         <v/>
       </c>
-      <c r="N28" s="37">
+      <c r="N28" s="43">
         <f>SUM(N8:N27)</f>
         <v/>
       </c>
-      <c r="O28" s="37">
+      <c r="O28" s="43">
         <f>SUM(O8:O27)</f>
         <v/>
       </c>
-      <c r="P28" s="37">
+      <c r="P28" s="43">
         <f>SUM(P8:P27)</f>
         <v/>
       </c>
-      <c r="Q28" s="37">
+      <c r="Q28" s="43">
         <f>SUM(Q8:Q27)</f>
         <v/>
       </c>
-      <c r="R28" s="37">
+      <c r="R28" s="43">
         <f>IFERROR(Q28/COUNTIF(E28:P28,"&gt;0"),0)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="8" customHeight="1">
-      <c r="B30" s="43" t="n"/>
+      <c r="B30" s="49" t="n"/>
     </row>
     <row r="31" ht="16" customHeight="1">
-      <c r="B31" s="44" t="inlineStr">
+      <c r="B31" s="50" t="inlineStr">
         <is>
           <t>MIX SHOP DIGITAL  ·  Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
     </row>
     <row r="32" ht="16" customHeight="1">
-      <c r="B32" s="45" t="inlineStr">
+      <c r="B32" s="51" t="inlineStr">
         <is>
           <t>Versión gratuita  ·  Más herramientas gratuitas para tu vida diaria  →  mixshopdigital.com.py</t>
         </is>
@@ -2908,7 +3138,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="ECF5"/>
-  <mergeCells count="12">
+  <mergeCells count="11">
     <mergeCell ref="B28:D28"/>
     <mergeCell ref="B32:R32"/>
     <mergeCell ref="B1:E1"/>
@@ -2919,7 +3149,6 @@
     <mergeCell ref="F2:R2"/>
     <mergeCell ref="C4:R4"/>
     <mergeCell ref="B2:E2"/>
-    <mergeCell ref="B3:R3"/>
     <mergeCell ref="B31:R31"/>
   </mergeCells>
   <conditionalFormatting sqref="F8:P27">
@@ -2964,6 +3193,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2986,671 +3216,676 @@
     <col width="16" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>MIX SHOP DIGITAL</t>
-        </is>
-      </c>
-      <c r="D1" s="2" t="inlineStr">
+    <row r="1" ht="38" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>VENCIMIENTOS</t>
         </is>
       </c>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>¿Qué tenés que pagar este mes?</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="4" customHeight="1">
-      <c r="B3" s="5" t="n"/>
+    <row r="3" ht="5" customHeight="1">
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="10" t="n"/>
+      <c r="G3" s="11" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="46" t="n"/>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="B4" s="52" t="n"/>
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Se arma solo con SERVICIOS: si ya cargaste el monto del mes figura como pagado; si no, te avisa cuándo vence.</t>
         </is>
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="14" t="inlineStr">
         <is>
           <t>←  Volver al PANEL</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>Anotar pagos</t>
         </is>
       </c>
     </row>
     <row r="7" ht="16" customHeight="1">
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>PAGADOS ESTE MES</t>
         </is>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="18" t="inlineStr">
         <is>
           <t>PENDIENTES</t>
         </is>
       </c>
-      <c r="F7" s="13" t="inlineStr">
+      <c r="F7" s="19" t="inlineStr">
         <is>
           <t>A PAGAR (APROX.)</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="B8" s="55">
+      <c r="B8" s="61">
         <f>COUNTIF(F11:F30,"✔*")</f>
         <v/>
       </c>
-      <c r="D8" s="56">
+      <c r="D8" s="62">
         <f>COUNTIF(B11:B30,"?*")-B8</f>
         <v/>
       </c>
-      <c r="F8" s="57">
+      <c r="F8" s="63">
         <f>SUMIF(F11:F30,"&lt;&gt;✔ Pagado",G11:G30)</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="15" customHeight="1">
-      <c r="B9" s="22">
+      <c r="B9" s="28">
         <f>"de "&amp;COUNTIF(B11:B30,"?*")&amp;" servicios"</f>
         <v/>
       </c>
-      <c r="D9" s="20" t="inlineStr">
+      <c r="D9" s="26" t="inlineStr">
         <is>
           <t>todavía sin pagar</t>
         </is>
       </c>
-      <c r="F9" s="21" t="inlineStr">
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>según tu promedio</t>
         </is>
       </c>
     </row>
     <row r="10" ht="24" customHeight="1">
-      <c r="B10" s="47" t="inlineStr">
+      <c r="B10" s="53" t="inlineStr">
         <is>
           <t>Servicio</t>
         </is>
       </c>
-      <c r="C10" s="47" t="inlineStr">
+      <c r="C10" s="53" t="inlineStr">
         <is>
           <t>Categoría</t>
         </is>
       </c>
-      <c r="D10" s="47" t="inlineStr">
+      <c r="D10" s="53" t="inlineStr">
         <is>
           <t>Vence</t>
         </is>
       </c>
-      <c r="E10" s="47" t="inlineStr">
+      <c r="E10" s="53" t="inlineStr">
         <is>
           <t>Pagaste este mes</t>
         </is>
       </c>
-      <c r="F10" s="47" t="inlineStr">
+      <c r="F10" s="53" t="inlineStr">
         <is>
           <t>Estado</t>
         </is>
       </c>
-      <c r="G10" s="47" t="inlineStr">
+      <c r="G10" s="53" t="inlineStr">
         <is>
           <t>Tu promedio</t>
         </is>
       </c>
     </row>
     <row r="11" ht="21" customHeight="1">
-      <c r="B11" s="28">
+      <c r="B11" s="34">
         <f>IF(SERVICIOS!B8="","",SERVICIOS!B8)</f>
         <v/>
       </c>
-      <c r="C11" s="58">
+      <c r="C11" s="64">
         <f>IF(B11="","",SERVICIOS!C8&amp;"")</f>
         <v/>
       </c>
-      <c r="D11" s="59">
+      <c r="D11" s="65">
         <f>IF(OR(B11="",N(SERVICIOS!D8)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D8,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E11" s="60">
+      <c r="E11" s="66">
         <f>IF(B11="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E8:P8,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F11" s="61">
+      <c r="F11" s="67">
         <f>IF(B11="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E11)&gt;0,"✔ Pagado",IF(D11="","Sin día de vencimiento",IF(D11&lt;TODAY(),"✖ Vencido",IF(D11=TODAY(),"⚠ Vence hoy",IF(D11-TODAY()&lt;=5,"⚠ Vence en "&amp;(D11-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G11" s="62">
+      <c r="G11" s="68">
         <f>IF(B11="","",SERVICIOS!R8)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="21" customHeight="1">
-      <c r="B12" s="32">
+      <c r="B12" s="38">
         <f>IF(SERVICIOS!B9="","",SERVICIOS!B9)</f>
         <v/>
       </c>
-      <c r="C12" s="63">
+      <c r="C12" s="69">
         <f>IF(B12="","",SERVICIOS!C9&amp;"")</f>
         <v/>
       </c>
-      <c r="D12" s="64">
+      <c r="D12" s="70">
         <f>IF(OR(B12="",N(SERVICIOS!D9)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D9,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E12" s="65">
+      <c r="E12" s="71">
         <f>IF(B12="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E9:P9,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F12" s="66">
+      <c r="F12" s="72">
         <f>IF(B12="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E12)&gt;0,"✔ Pagado",IF(D12="","Sin día de vencimiento",IF(D12&lt;TODAY(),"✖ Vencido",IF(D12=TODAY(),"⚠ Vence hoy",IF(D12-TODAY()&lt;=5,"⚠ Vence en "&amp;(D12-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G12" s="67">
+      <c r="G12" s="73">
         <f>IF(B12="","",SERVICIOS!R9)</f>
         <v/>
       </c>
     </row>
     <row r="13" ht="21" customHeight="1">
-      <c r="B13" s="28">
+      <c r="B13" s="34">
         <f>IF(SERVICIOS!B10="","",SERVICIOS!B10)</f>
         <v/>
       </c>
-      <c r="C13" s="58">
+      <c r="C13" s="64">
         <f>IF(B13="","",SERVICIOS!C10&amp;"")</f>
         <v/>
       </c>
-      <c r="D13" s="59">
+      <c r="D13" s="65">
         <f>IF(OR(B13="",N(SERVICIOS!D10)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D10,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E13" s="60">
+      <c r="E13" s="66">
         <f>IF(B13="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E10:P10,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F13" s="61">
+      <c r="F13" s="67">
         <f>IF(B13="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E13)&gt;0,"✔ Pagado",IF(D13="","Sin día de vencimiento",IF(D13&lt;TODAY(),"✖ Vencido",IF(D13=TODAY(),"⚠ Vence hoy",IF(D13-TODAY()&lt;=5,"⚠ Vence en "&amp;(D13-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G13" s="62">
+      <c r="G13" s="68">
         <f>IF(B13="","",SERVICIOS!R10)</f>
         <v/>
       </c>
     </row>
     <row r="14" ht="21" customHeight="1">
-      <c r="B14" s="32">
+      <c r="B14" s="38">
         <f>IF(SERVICIOS!B11="","",SERVICIOS!B11)</f>
         <v/>
       </c>
-      <c r="C14" s="63">
+      <c r="C14" s="69">
         <f>IF(B14="","",SERVICIOS!C11&amp;"")</f>
         <v/>
       </c>
-      <c r="D14" s="64">
+      <c r="D14" s="70">
         <f>IF(OR(B14="",N(SERVICIOS!D11)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D11,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E14" s="65">
+      <c r="E14" s="71">
         <f>IF(B14="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E11:P11,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F14" s="66">
+      <c r="F14" s="72">
         <f>IF(B14="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E14)&gt;0,"✔ Pagado",IF(D14="","Sin día de vencimiento",IF(D14&lt;TODAY(),"✖ Vencido",IF(D14=TODAY(),"⚠ Vence hoy",IF(D14-TODAY()&lt;=5,"⚠ Vence en "&amp;(D14-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G14" s="67">
+      <c r="G14" s="73">
         <f>IF(B14="","",SERVICIOS!R11)</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="21" customHeight="1">
-      <c r="B15" s="28">
+      <c r="B15" s="34">
         <f>IF(SERVICIOS!B12="","",SERVICIOS!B12)</f>
         <v/>
       </c>
-      <c r="C15" s="58">
+      <c r="C15" s="64">
         <f>IF(B15="","",SERVICIOS!C12&amp;"")</f>
         <v/>
       </c>
-      <c r="D15" s="59">
+      <c r="D15" s="65">
         <f>IF(OR(B15="",N(SERVICIOS!D12)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D12,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E15" s="60">
+      <c r="E15" s="66">
         <f>IF(B15="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E12:P12,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F15" s="61">
+      <c r="F15" s="67">
         <f>IF(B15="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E15)&gt;0,"✔ Pagado",IF(D15="","Sin día de vencimiento",IF(D15&lt;TODAY(),"✖ Vencido",IF(D15=TODAY(),"⚠ Vence hoy",IF(D15-TODAY()&lt;=5,"⚠ Vence en "&amp;(D15-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G15" s="62">
+      <c r="G15" s="68">
         <f>IF(B15="","",SERVICIOS!R12)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="21" customHeight="1">
-      <c r="B16" s="32">
+      <c r="B16" s="38">
         <f>IF(SERVICIOS!B13="","",SERVICIOS!B13)</f>
         <v/>
       </c>
-      <c r="C16" s="63">
+      <c r="C16" s="69">
         <f>IF(B16="","",SERVICIOS!C13&amp;"")</f>
         <v/>
       </c>
-      <c r="D16" s="64">
+      <c r="D16" s="70">
         <f>IF(OR(B16="",N(SERVICIOS!D13)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D13,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E16" s="65">
+      <c r="E16" s="71">
         <f>IF(B16="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E13:P13,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F16" s="66">
+      <c r="F16" s="72">
         <f>IF(B16="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E16)&gt;0,"✔ Pagado",IF(D16="","Sin día de vencimiento",IF(D16&lt;TODAY(),"✖ Vencido",IF(D16=TODAY(),"⚠ Vence hoy",IF(D16-TODAY()&lt;=5,"⚠ Vence en "&amp;(D16-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G16" s="67">
+      <c r="G16" s="73">
         <f>IF(B16="","",SERVICIOS!R13)</f>
         <v/>
       </c>
     </row>
     <row r="17" ht="21" customHeight="1">
-      <c r="B17" s="28">
+      <c r="B17" s="34">
         <f>IF(SERVICIOS!B14="","",SERVICIOS!B14)</f>
         <v/>
       </c>
-      <c r="C17" s="58">
+      <c r="C17" s="64">
         <f>IF(B17="","",SERVICIOS!C14&amp;"")</f>
         <v/>
       </c>
-      <c r="D17" s="59">
+      <c r="D17" s="65">
         <f>IF(OR(B17="",N(SERVICIOS!D14)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D14,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E17" s="60">
+      <c r="E17" s="66">
         <f>IF(B17="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E14:P14,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F17" s="61">
+      <c r="F17" s="67">
         <f>IF(B17="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E17)&gt;0,"✔ Pagado",IF(D17="","Sin día de vencimiento",IF(D17&lt;TODAY(),"✖ Vencido",IF(D17=TODAY(),"⚠ Vence hoy",IF(D17-TODAY()&lt;=5,"⚠ Vence en "&amp;(D17-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G17" s="62">
+      <c r="G17" s="68">
         <f>IF(B17="","",SERVICIOS!R14)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="21" customHeight="1">
-      <c r="B18" s="32">
+      <c r="B18" s="38">
         <f>IF(SERVICIOS!B15="","",SERVICIOS!B15)</f>
         <v/>
       </c>
-      <c r="C18" s="63">
+      <c r="C18" s="69">
         <f>IF(B18="","",SERVICIOS!C15&amp;"")</f>
         <v/>
       </c>
-      <c r="D18" s="64">
+      <c r="D18" s="70">
         <f>IF(OR(B18="",N(SERVICIOS!D15)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D15,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E18" s="65">
+      <c r="E18" s="71">
         <f>IF(B18="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E15:P15,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F18" s="66">
+      <c r="F18" s="72">
         <f>IF(B18="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E18)&gt;0,"✔ Pagado",IF(D18="","Sin día de vencimiento",IF(D18&lt;TODAY(),"✖ Vencido",IF(D18=TODAY(),"⚠ Vence hoy",IF(D18-TODAY()&lt;=5,"⚠ Vence en "&amp;(D18-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G18" s="67">
+      <c r="G18" s="73">
         <f>IF(B18="","",SERVICIOS!R15)</f>
         <v/>
       </c>
     </row>
     <row r="19" ht="21" customHeight="1">
-      <c r="B19" s="28">
+      <c r="B19" s="34">
         <f>IF(SERVICIOS!B16="","",SERVICIOS!B16)</f>
         <v/>
       </c>
-      <c r="C19" s="58">
+      <c r="C19" s="64">
         <f>IF(B19="","",SERVICIOS!C16&amp;"")</f>
         <v/>
       </c>
-      <c r="D19" s="59">
+      <c r="D19" s="65">
         <f>IF(OR(B19="",N(SERVICIOS!D16)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D16,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E19" s="60">
+      <c r="E19" s="66">
         <f>IF(B19="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E16:P16,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F19" s="61">
+      <c r="F19" s="67">
         <f>IF(B19="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E19)&gt;0,"✔ Pagado",IF(D19="","Sin día de vencimiento",IF(D19&lt;TODAY(),"✖ Vencido",IF(D19=TODAY(),"⚠ Vence hoy",IF(D19-TODAY()&lt;=5,"⚠ Vence en "&amp;(D19-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G19" s="62">
+      <c r="G19" s="68">
         <f>IF(B19="","",SERVICIOS!R16)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="21" customHeight="1">
-      <c r="B20" s="32">
+      <c r="B20" s="38">
         <f>IF(SERVICIOS!B17="","",SERVICIOS!B17)</f>
         <v/>
       </c>
-      <c r="C20" s="63">
+      <c r="C20" s="69">
         <f>IF(B20="","",SERVICIOS!C17&amp;"")</f>
         <v/>
       </c>
-      <c r="D20" s="64">
+      <c r="D20" s="70">
         <f>IF(OR(B20="",N(SERVICIOS!D17)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D17,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E20" s="65">
+      <c r="E20" s="71">
         <f>IF(B20="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E17:P17,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F20" s="66">
+      <c r="F20" s="72">
         <f>IF(B20="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E20)&gt;0,"✔ Pagado",IF(D20="","Sin día de vencimiento",IF(D20&lt;TODAY(),"✖ Vencido",IF(D20=TODAY(),"⚠ Vence hoy",IF(D20-TODAY()&lt;=5,"⚠ Vence en "&amp;(D20-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G20" s="67">
+      <c r="G20" s="73">
         <f>IF(B20="","",SERVICIOS!R17)</f>
         <v/>
       </c>
     </row>
     <row r="21" ht="21" customHeight="1">
-      <c r="B21" s="28">
+      <c r="B21" s="34">
         <f>IF(SERVICIOS!B18="","",SERVICIOS!B18)</f>
         <v/>
       </c>
-      <c r="C21" s="58">
+      <c r="C21" s="64">
         <f>IF(B21="","",SERVICIOS!C18&amp;"")</f>
         <v/>
       </c>
-      <c r="D21" s="59">
+      <c r="D21" s="65">
         <f>IF(OR(B21="",N(SERVICIOS!D18)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D18,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E21" s="60">
+      <c r="E21" s="66">
         <f>IF(B21="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E18:P18,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F21" s="61">
+      <c r="F21" s="67">
         <f>IF(B21="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E21)&gt;0,"✔ Pagado",IF(D21="","Sin día de vencimiento",IF(D21&lt;TODAY(),"✖ Vencido",IF(D21=TODAY(),"⚠ Vence hoy",IF(D21-TODAY()&lt;=5,"⚠ Vence en "&amp;(D21-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G21" s="62">
+      <c r="G21" s="68">
         <f>IF(B21="","",SERVICIOS!R18)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="21" customHeight="1">
-      <c r="B22" s="32">
+      <c r="B22" s="38">
         <f>IF(SERVICIOS!B19="","",SERVICIOS!B19)</f>
         <v/>
       </c>
-      <c r="C22" s="63">
+      <c r="C22" s="69">
         <f>IF(B22="","",SERVICIOS!C19&amp;"")</f>
         <v/>
       </c>
-      <c r="D22" s="64">
+      <c r="D22" s="70">
         <f>IF(OR(B22="",N(SERVICIOS!D19)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D19,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E22" s="65">
+      <c r="E22" s="71">
         <f>IF(B22="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E19:P19,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F22" s="66">
+      <c r="F22" s="72">
         <f>IF(B22="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E22)&gt;0,"✔ Pagado",IF(D22="","Sin día de vencimiento",IF(D22&lt;TODAY(),"✖ Vencido",IF(D22=TODAY(),"⚠ Vence hoy",IF(D22-TODAY()&lt;=5,"⚠ Vence en "&amp;(D22-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G22" s="67">
+      <c r="G22" s="73">
         <f>IF(B22="","",SERVICIOS!R19)</f>
         <v/>
       </c>
     </row>
     <row r="23" ht="21" customHeight="1">
-      <c r="B23" s="28">
+      <c r="B23" s="34">
         <f>IF(SERVICIOS!B20="","",SERVICIOS!B20)</f>
         <v/>
       </c>
-      <c r="C23" s="58">
+      <c r="C23" s="64">
         <f>IF(B23="","",SERVICIOS!C20&amp;"")</f>
         <v/>
       </c>
-      <c r="D23" s="59">
+      <c r="D23" s="65">
         <f>IF(OR(B23="",N(SERVICIOS!D20)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D20,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E23" s="60">
+      <c r="E23" s="66">
         <f>IF(B23="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E20:P20,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F23" s="61">
+      <c r="F23" s="67">
         <f>IF(B23="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E23)&gt;0,"✔ Pagado",IF(D23="","Sin día de vencimiento",IF(D23&lt;TODAY(),"✖ Vencido",IF(D23=TODAY(),"⚠ Vence hoy",IF(D23-TODAY()&lt;=5,"⚠ Vence en "&amp;(D23-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G23" s="62">
+      <c r="G23" s="68">
         <f>IF(B23="","",SERVICIOS!R20)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="21" customHeight="1">
-      <c r="B24" s="32">
+      <c r="B24" s="38">
         <f>IF(SERVICIOS!B21="","",SERVICIOS!B21)</f>
         <v/>
       </c>
-      <c r="C24" s="63">
+      <c r="C24" s="69">
         <f>IF(B24="","",SERVICIOS!C21&amp;"")</f>
         <v/>
       </c>
-      <c r="D24" s="64">
+      <c r="D24" s="70">
         <f>IF(OR(B24="",N(SERVICIOS!D21)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D21,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E24" s="65">
+      <c r="E24" s="71">
         <f>IF(B24="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E21:P21,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F24" s="66">
+      <c r="F24" s="72">
         <f>IF(B24="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E24)&gt;0,"✔ Pagado",IF(D24="","Sin día de vencimiento",IF(D24&lt;TODAY(),"✖ Vencido",IF(D24=TODAY(),"⚠ Vence hoy",IF(D24-TODAY()&lt;=5,"⚠ Vence en "&amp;(D24-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G24" s="67">
+      <c r="G24" s="73">
         <f>IF(B24="","",SERVICIOS!R21)</f>
         <v/>
       </c>
     </row>
     <row r="25" ht="21" customHeight="1">
-      <c r="B25" s="28">
+      <c r="B25" s="34">
         <f>IF(SERVICIOS!B22="","",SERVICIOS!B22)</f>
         <v/>
       </c>
-      <c r="C25" s="58">
+      <c r="C25" s="64">
         <f>IF(B25="","",SERVICIOS!C22&amp;"")</f>
         <v/>
       </c>
-      <c r="D25" s="59">
+      <c r="D25" s="65">
         <f>IF(OR(B25="",N(SERVICIOS!D22)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D22,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E25" s="60">
+      <c r="E25" s="66">
         <f>IF(B25="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E22:P22,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F25" s="61">
+      <c r="F25" s="67">
         <f>IF(B25="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E25)&gt;0,"✔ Pagado",IF(D25="","Sin día de vencimiento",IF(D25&lt;TODAY(),"✖ Vencido",IF(D25=TODAY(),"⚠ Vence hoy",IF(D25-TODAY()&lt;=5,"⚠ Vence en "&amp;(D25-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G25" s="62">
+      <c r="G25" s="68">
         <f>IF(B25="","",SERVICIOS!R22)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="21" customHeight="1">
-      <c r="B26" s="32">
+      <c r="B26" s="38">
         <f>IF(SERVICIOS!B23="","",SERVICIOS!B23)</f>
         <v/>
       </c>
-      <c r="C26" s="63">
+      <c r="C26" s="69">
         <f>IF(B26="","",SERVICIOS!C23&amp;"")</f>
         <v/>
       </c>
-      <c r="D26" s="64">
+      <c r="D26" s="70">
         <f>IF(OR(B26="",N(SERVICIOS!D23)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D23,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E26" s="65">
+      <c r="E26" s="71">
         <f>IF(B26="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E23:P23,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F26" s="66">
+      <c r="F26" s="72">
         <f>IF(B26="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E26)&gt;0,"✔ Pagado",IF(D26="","Sin día de vencimiento",IF(D26&lt;TODAY(),"✖ Vencido",IF(D26=TODAY(),"⚠ Vence hoy",IF(D26-TODAY()&lt;=5,"⚠ Vence en "&amp;(D26-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G26" s="67">
+      <c r="G26" s="73">
         <f>IF(B26="","",SERVICIOS!R23)</f>
         <v/>
       </c>
     </row>
     <row r="27" ht="21" customHeight="1">
-      <c r="B27" s="28">
+      <c r="B27" s="34">
         <f>IF(SERVICIOS!B24="","",SERVICIOS!B24)</f>
         <v/>
       </c>
-      <c r="C27" s="58">
+      <c r="C27" s="64">
         <f>IF(B27="","",SERVICIOS!C24&amp;"")</f>
         <v/>
       </c>
-      <c r="D27" s="59">
+      <c r="D27" s="65">
         <f>IF(OR(B27="",N(SERVICIOS!D24)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D24,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E27" s="60">
+      <c r="E27" s="66">
         <f>IF(B27="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E24:P24,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F27" s="61">
+      <c r="F27" s="67">
         <f>IF(B27="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E27)&gt;0,"✔ Pagado",IF(D27="","Sin día de vencimiento",IF(D27&lt;TODAY(),"✖ Vencido",IF(D27=TODAY(),"⚠ Vence hoy",IF(D27-TODAY()&lt;=5,"⚠ Vence en "&amp;(D27-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G27" s="62">
+      <c r="G27" s="68">
         <f>IF(B27="","",SERVICIOS!R24)</f>
         <v/>
       </c>
     </row>
     <row r="28" ht="21" customHeight="1">
-      <c r="B28" s="32">
+      <c r="B28" s="38">
         <f>IF(SERVICIOS!B25="","",SERVICIOS!B25)</f>
         <v/>
       </c>
-      <c r="C28" s="63">
+      <c r="C28" s="69">
         <f>IF(B28="","",SERVICIOS!C25&amp;"")</f>
         <v/>
       </c>
-      <c r="D28" s="64">
+      <c r="D28" s="70">
         <f>IF(OR(B28="",N(SERVICIOS!D25)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D25,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E28" s="65">
+      <c r="E28" s="71">
         <f>IF(B28="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E25:P25,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F28" s="66">
+      <c r="F28" s="72">
         <f>IF(B28="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E28)&gt;0,"✔ Pagado",IF(D28="","Sin día de vencimiento",IF(D28&lt;TODAY(),"✖ Vencido",IF(D28=TODAY(),"⚠ Vence hoy",IF(D28-TODAY()&lt;=5,"⚠ Vence en "&amp;(D28-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G28" s="67">
+      <c r="G28" s="73">
         <f>IF(B28="","",SERVICIOS!R25)</f>
         <v/>
       </c>
     </row>
     <row r="29" ht="21" customHeight="1">
-      <c r="B29" s="28">
+      <c r="B29" s="34">
         <f>IF(SERVICIOS!B26="","",SERVICIOS!B26)</f>
         <v/>
       </c>
-      <c r="C29" s="58">
+      <c r="C29" s="64">
         <f>IF(B29="","",SERVICIOS!C26&amp;"")</f>
         <v/>
       </c>
-      <c r="D29" s="59">
+      <c r="D29" s="65">
         <f>IF(OR(B29="",N(SERVICIOS!D26)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D26,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E29" s="60">
+      <c r="E29" s="66">
         <f>IF(B29="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E26:P26,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F29" s="61">
+      <c r="F29" s="67">
         <f>IF(B29="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E29)&gt;0,"✔ Pagado",IF(D29="","Sin día de vencimiento",IF(D29&lt;TODAY(),"✖ Vencido",IF(D29=TODAY(),"⚠ Vence hoy",IF(D29-TODAY()&lt;=5,"⚠ Vence en "&amp;(D29-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G29" s="62">
+      <c r="G29" s="68">
         <f>IF(B29="","",SERVICIOS!R26)</f>
         <v/>
       </c>
     </row>
     <row r="30" ht="21" customHeight="1">
-      <c r="B30" s="32">
+      <c r="B30" s="38">
         <f>IF(SERVICIOS!B27="","",SERVICIOS!B27)</f>
         <v/>
       </c>
-      <c r="C30" s="63">
+      <c r="C30" s="69">
         <f>IF(B30="","",SERVICIOS!C27&amp;"")</f>
         <v/>
       </c>
-      <c r="D30" s="64">
+      <c r="D30" s="70">
         <f>IF(OR(B30="",N(SERVICIOS!D27)=0),"",DATE(YEAR(TODAY()),MONTH(TODAY()),MIN(SERVICIOS!D27,DAY(DATE(YEAR(TODAY()),MONTH(TODAY())+1,0)))))</f>
         <v/>
       </c>
-      <c r="E30" s="65">
+      <c r="E30" s="71">
         <f>IF(B30="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"",INDEX(SERVICIOS!E27:P27,MONTH(TODAY()))))</f>
         <v/>
       </c>
-      <c r="F30" s="66">
+      <c r="F30" s="72">
         <f>IF(B30="","",IF(YEAR(TODAY())&lt;&gt;AnioCtl,"Cambiá el año en AJUSTES",IF(N(E30)&gt;0,"✔ Pagado",IF(D30="","Sin día de vencimiento",IF(D30&lt;TODAY(),"✖ Vencido",IF(D30=TODAY(),"⚠ Vence hoy",IF(D30-TODAY()&lt;=5,"⚠ Vence en "&amp;(D30-TODAY())&amp;" día(s)","Pendiente")))))))</f>
         <v/>
       </c>
-      <c r="G30" s="67">
+      <c r="G30" s="73">
         <f>IF(B30="","",SERVICIOS!R27)</f>
         <v/>
       </c>
     </row>
     <row r="31">
-      <c r="B31" s="68" t="inlineStr">
+      <c r="B31" s="74" t="inlineStr">
         <is>
           <t>El «promedio» es lo que pagás en promedio por mes: sirve para estimar cuánto te falta pagar. Es una referencia, no el monto exacto de la factura.</t>
         </is>
       </c>
     </row>
     <row r="33" ht="8" customHeight="1">
-      <c r="B33" s="43" t="n"/>
+      <c r="B33" s="49" t="n"/>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="44" t="inlineStr">
+      <c r="B34" s="50" t="inlineStr">
         <is>
           <t>MIX SHOP DIGITAL  ·  Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
     </row>
     <row r="35" ht="16" customHeight="1">
-      <c r="B35" s="45" t="inlineStr">
+      <c r="B35" s="51" t="inlineStr">
         <is>
           <t>Versión gratuita  ·  Más herramientas gratuitas para tu vida diaria  →  mixshopdigital.com.py</t>
         </is>
@@ -3658,7 +3893,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="ECF5"/>
-  <mergeCells count="21">
+  <mergeCells count="20">
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="F7:G7"/>
     <mergeCell ref="B34:G34"/>
@@ -3675,7 +3910,6 @@
     <mergeCell ref="D2:G2"/>
     <mergeCell ref="D9:E9"/>
     <mergeCell ref="F9:G9"/>
-    <mergeCell ref="B3:G3"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="B5:C5"/>
     <mergeCell ref="B31:G31"/>
@@ -3708,6 +3942,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3727,203 +3962,202 @@
     <col width="56" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>MIX SHOP DIGITAL</t>
-        </is>
-      </c>
-      <c r="C1" s="2" t="inlineStr">
+    <row r="1" ht="38" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>AJUSTES</t>
         </is>
       </c>
+      <c r="D1" s="2" t="n"/>
     </row>
     <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="3" t="inlineStr">
+      <c r="B2" s="4" t="inlineStr">
         <is>
           <t>Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
-      <c r="C2" s="4" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Cargalos una sola vez</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="4" customHeight="1">
-      <c r="B3" s="5" t="n"/>
+    <row r="3" ht="5" customHeight="1">
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="8" t="n"/>
+      <c r="D3" s="10" t="n"/>
     </row>
     <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="46" t="inlineStr">
+      <c r="B4" s="52" t="inlineStr">
         <is>
           <t>← VOLVER</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="12" t="inlineStr">
         <is>
           <t>Completá solamente las celdas amarillas. Estos datos alimentan las demás hojas automáticamente.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="26" t="inlineStr">
+      <c r="B6" s="32" t="inlineStr">
         <is>
           <t>1. TU HOGAR</t>
         </is>
       </c>
     </row>
     <row r="7" ht="28" customHeight="1">
-      <c r="B7" s="69" t="inlineStr">
+      <c r="B7" s="75" t="inlineStr">
         <is>
           <t>Nombre del hogar</t>
         </is>
       </c>
-      <c r="C7" s="70" t="inlineStr">
+      <c r="C7" s="76" t="inlineStr">
         <is>
           <t>Mi hogar</t>
         </is>
       </c>
-      <c r="D7" s="71" t="inlineStr">
+      <c r="D7" s="77" t="inlineStr">
         <is>
           <t>Aparece en el PANEL.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="28" customHeight="1">
-      <c r="B8" s="69" t="inlineStr">
+      <c r="B8" s="75" t="inlineStr">
         <is>
           <t>Año a controlar</t>
         </is>
       </c>
-      <c r="C8" s="72" t="n">
+      <c r="C8" s="78" t="n">
         <v>2026</v>
       </c>
-      <c r="D8" s="71" t="inlineStr">
+      <c r="D8" s="77" t="inlineStr">
         <is>
           <t>El PANEL y SERVICIOS muestran los 12 meses de este año.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="28" customHeight="1">
-      <c r="B9" s="69" t="inlineStr">
+      <c r="B9" s="75" t="inlineStr">
         <is>
           <t>Moneda</t>
         </is>
       </c>
-      <c r="C9" s="70" t="inlineStr">
+      <c r="C9" s="76" t="inlineStr">
         <is>
           <t>Gs.</t>
         </is>
       </c>
-      <c r="D9" s="71" t="inlineStr">
+      <c r="D9" s="77" t="inlineStr">
         <is>
           <t>Símbolo que se muestra en las hojas.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="28" customHeight="1">
-      <c r="B10" s="69" t="inlineStr">
+      <c r="B10" s="75" t="inlineStr">
         <is>
           <t>Presupuesto mensual del hogar</t>
         </is>
       </c>
-      <c r="C10" s="73" t="n">
+      <c r="C10" s="79" t="n">
         <v>0</v>
       </c>
-      <c r="D10" s="71" t="inlineStr">
+      <c r="D10" s="77" t="inlineStr">
         <is>
           <t>Cuánto querés gastar como máximo por mes en estos servicios y gastos fijos. Si no tenés, dejalo en 0.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="38" t="inlineStr">
+      <c r="B12" s="44" t="inlineStr">
         <is>
           <t>2. CATEGORÍAS (podés renombrarlas)</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="6" t="inlineStr">
+      <c r="B13" s="12" t="inlineStr">
         <is>
           <t>Se usan en la lista desplegable de SERVICIOS. Cambiá el nombre, pero no dejes huecos entre medio.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="70" t="inlineStr">
+      <c r="B14" s="76" t="inlineStr">
         <is>
           <t>Servicios básicos</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
+      <c r="C14" s="12" t="inlineStr">
         <is>
           <t>Hasta 8 categorías.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="70" t="inlineStr">
+      <c r="B15" s="76" t="inlineStr">
         <is>
           <t>Comunicaciones</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="70" t="inlineStr">
+      <c r="B16" s="76" t="inlineStr">
         <is>
           <t>Vivienda</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="70" t="inlineStr">
+      <c r="B17" s="76" t="inlineStr">
         <is>
           <t>Educación</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="70" t="inlineStr">
+      <c r="B18" s="76" t="inlineStr">
         <is>
           <t>Salud</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="70" t="inlineStr">
+      <c r="B19" s="76" t="inlineStr">
         <is>
           <t>Seguros</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="70" t="inlineStr">
+      <c r="B20" s="76" t="inlineStr">
         <is>
           <t>Transporte</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="70" t="inlineStr">
+      <c r="B21" s="76" t="inlineStr">
         <is>
           <t>Otros</t>
         </is>
       </c>
     </row>
     <row r="24" ht="8" customHeight="1">
-      <c r="B24" s="43" t="n"/>
+      <c r="B24" s="49" t="n"/>
     </row>
     <row r="25" ht="16" customHeight="1">
-      <c r="B25" s="44" t="inlineStr">
+      <c r="B25" s="50" t="inlineStr">
         <is>
           <t>MIX SHOP DIGITAL  ·  Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="16" customHeight="1">
-      <c r="B26" s="45" t="inlineStr">
+      <c r="B26" s="51" t="inlineStr">
         <is>
           <t>Versión gratuita  ·  Más herramientas gratuitas para tu vida diaria  →  mixshopdigital.com.py</t>
         </is>
@@ -3931,8 +4165,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="ECF5"/>
-  <mergeCells count="9">
-    <mergeCell ref="B3:D3"/>
+  <mergeCells count="8">
     <mergeCell ref="C2:D2"/>
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="B26:D26"/>
@@ -3969,6 +4202,7 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -3992,197 +4226,204 @@
     <col width="16" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="B1" s="1" t="inlineStr">
+    <row r="1" ht="38" customHeight="1">
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="2" t="n"/>
+      <c r="D1" s="3" t="inlineStr">
+        <is>
+          <t>AYUDA</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="n"/>
+      <c r="F1" s="2" t="n"/>
+      <c r="G1" s="2" t="n"/>
+      <c r="H1" s="2" t="n"/>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="B2" s="4" t="inlineStr">
+        <is>
+          <t>Herramientas inteligentes que simplifican tu vida.</t>
+        </is>
+      </c>
+      <c r="D2" s="5" t="inlineStr">
+        <is>
+          <t>Se aprende en 2 minutos</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="5" customHeight="1">
+      <c r="B3" s="6" t="n"/>
+      <c r="C3" s="7" t="n"/>
+      <c r="D3" s="8" t="n"/>
+      <c r="E3" s="9" t="n"/>
+      <c r="F3" s="9" t="n"/>
+      <c r="G3" s="10" t="n"/>
+      <c r="H3" s="11" t="n"/>
+    </row>
+    <row r="4" ht="20" customHeight="1">
+      <c r="B4" s="52" t="inlineStr">
+        <is>
+          <t>← VOLVER</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Leé esta hoja una vez. Después ya no la vas a necesitar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>¿PARA QUÉ SIRVE?</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="33" customHeight="1">
+      <c r="B7" s="80" t="inlineStr">
+        <is>
+          <t>Para tener a mano cuánto pagás de agua, luz, internet, cable y demás gastos fijos del hogar, mes por mes, y no olvidarte de ningún vencimiento. Sin fórmulas y sin Internet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="44" t="inlineStr">
+        <is>
+          <t>EMPEZÁ EN 3 PASOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18.5" customHeight="1">
+      <c r="B10" s="80" t="inlineStr">
+        <is>
+          <t>1) En AJUSTES poné el nombre de tu hogar, el año y, si querés, tu presupuesto mensual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="33" customHeight="1">
+      <c r="B11" s="80" t="inlineStr">
+        <is>
+          <t>2) En SERVICIOS revisá la lista (podés cambiar los nombres y agregar más), poné el día de vencimiento de cada uno y escribí cuánto pagaste cada mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18.5" customHeight="1">
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t>3) Mirá el PANEL para ver tus gastos y VENCIMIENTOS para saber qué te falta pagar este mes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>COLORES Y AVISOS</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="47.5" customHeight="1">
+      <c r="B15" s="80" t="inlineStr">
+        <is>
+          <t>Amarillo claro: celdas que completás vos.   Gris o blanco: se calcula solo (bloqueado).   Naranja en SERVICIOS: el monto subió más de 20 % respecto del mes anterior.   En VENCIMIENTOS: verde pagado, naranja por vencer, rojo vencido.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="44" t="inlineStr">
+        <is>
+          <t>PREGUNTAS FRECUENTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18.5" customHeight="1">
+      <c r="B18" s="80" t="inlineStr">
+        <is>
+          <t>• Veo todo en cero: hacé clic en «Habilitar edición» en la barra amarilla de Excel.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="33" customHeight="1">
+      <c r="B19" s="80" t="inlineStr">
+        <is>
+          <t>• ¿Cómo marco un servicio como pagado? Escribí el monto pagado en la columna del mes. Mientras esté vacío, figura como pendiente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="18.5" customHeight="1">
+      <c r="B20" s="80" t="inlineStr">
+        <is>
+          <t>• ¿Cómo agrego un servicio? Escribí su nombre en una fila libre de SERVICIOS (hay 20 filas).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18.5" customHeight="1">
+      <c r="B21" s="80" t="inlineStr">
+        <is>
+          <t>• ¿Por qué VENCIMIENTOS dice «Cambiá el año en AJUSTES»? Porque el año de control no es el año actual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="33" customHeight="1">
+      <c r="B22" s="80" t="inlineStr">
+        <is>
+          <t>• ¿Qué es el «promedio»? Lo que pagás en promedio por mes en ese servicio; sirve para estimar cuánto te falta pagar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="33" customHeight="1">
+      <c r="B23" s="80" t="inlineStr">
+        <is>
+          <t>• Solo se editan las celdas amarillas: el resto está protegido para que no se rompan las fórmulas por accidente.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="44" t="inlineStr">
+        <is>
+          <t>SOBRE LA PROTECCIÓN</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="18.5" customHeight="1">
+      <c r="B26" s="80" t="inlineStr">
+        <is>
+          <t>La protección de Excel evita borrados accidentales, pero no es un sistema de seguridad criptográfico.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="81" t="inlineStr">
         <is>
           <t>MIX SHOP DIGITAL</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
-        <is>
-          <t>AYUDA</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>Herramientas inteligentes que simplifican tu vida.</t>
-        </is>
-      </c>
-      <c r="D2" s="4" t="inlineStr">
-        <is>
-          <t>Se aprende en 2 minutos</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="4" customHeight="1">
-      <c r="B3" s="5" t="n"/>
-    </row>
-    <row r="4" ht="20" customHeight="1">
-      <c r="B4" s="46" t="inlineStr">
-        <is>
-          <t>← VOLVER</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>Leé esta hoja una vez. Después ya no la vas a necesitar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="B6" s="26" t="inlineStr">
-        <is>
-          <t>¿PARA QUÉ SIRVE?</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="33" customHeight="1">
-      <c r="B7" s="74" t="inlineStr">
-        <is>
-          <t>Para tener a mano cuánto pagás de agua, luz, internet, cable y demás gastos fijos del hogar, mes por mes, y no olvidarte de ningún vencimiento. Sin fórmulas y sin Internet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="38" t="inlineStr">
-        <is>
-          <t>EMPEZÁ EN 3 PASOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="18.5" customHeight="1">
-      <c r="B10" s="74" t="inlineStr">
-        <is>
-          <t>1) En AJUSTES poné el nombre de tu hogar, el año y, si querés, tu presupuesto mensual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="33" customHeight="1">
-      <c r="B11" s="74" t="inlineStr">
-        <is>
-          <t>2) En SERVICIOS revisá la lista (podés cambiar los nombres y agregar más), poné el día de vencimiento de cada uno y escribí cuánto pagaste cada mes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18.5" customHeight="1">
-      <c r="B12" s="74" t="inlineStr">
-        <is>
-          <t>3) Mirá el PANEL para ver tus gastos y VENCIMIENTOS para saber qué te falta pagar este mes.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="26" t="inlineStr">
-        <is>
-          <t>COLORES Y AVISOS</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="47.5" customHeight="1">
-      <c r="B15" s="74" t="inlineStr">
-        <is>
-          <t>Amarillo claro: celdas que completás vos.   Gris o blanco: se calcula solo (bloqueado).   Naranja en SERVICIOS: el monto subió más de 20 % respecto del mes anterior.   En VENCIMIENTOS: verde pagado, naranja por vencer, rojo vencido.</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="38" t="inlineStr">
-        <is>
-          <t>PREGUNTAS FRECUENTES</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="18.5" customHeight="1">
-      <c r="B18" s="74" t="inlineStr">
-        <is>
-          <t>• Veo todo en cero: hacé clic en «Habilitar edición» en la barra amarilla de Excel.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="33" customHeight="1">
-      <c r="B19" s="74" t="inlineStr">
-        <is>
-          <t>• ¿Cómo marco un servicio como pagado? Escribí el monto pagado en la columna del mes. Mientras esté vacío, figura como pendiente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="18.5" customHeight="1">
-      <c r="B20" s="74" t="inlineStr">
-        <is>
-          <t>• ¿Cómo agrego un servicio? Escribí su nombre en una fila libre de SERVICIOS (hay 20 filas).</t>
-        </is>
-      </c>
-    </row>
-    <row r="21" ht="18.5" customHeight="1">
-      <c r="B21" s="74" t="inlineStr">
-        <is>
-          <t>• ¿Por qué VENCIMIENTOS dice «Cambiá el año en AJUSTES»? Porque el año de control no es el año actual.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="33" customHeight="1">
-      <c r="B22" s="74" t="inlineStr">
-        <is>
-          <t>• ¿Qué es el «promedio»? Lo que pagás en promedio por mes en ese servicio; sirve para estimar cuánto te falta pagar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="33" customHeight="1">
-      <c r="B23" s="74" t="inlineStr">
-        <is>
-          <t>• Solo se editan las celdas amarillas: el resto está protegido para que no se rompan las fórmulas por accidente.</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="38" t="inlineStr">
-        <is>
-          <t>SOBRE LA PROTECCIÓN</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="18.5" customHeight="1">
-      <c r="B26" s="74" t="inlineStr">
-        <is>
-          <t>La protección de Excel evita borrados accidentales, pero no es un sistema de seguridad criptográfico.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="75" t="inlineStr">
-        <is>
-          <t>MIX SHOP DIGITAL</t>
-        </is>
-      </c>
     </row>
     <row r="29" ht="33" customHeight="1">
-      <c r="B29" s="74" t="inlineStr">
+      <c r="B29" s="80" t="inlineStr">
         <is>
           <t>Esta planilla es una herramienta gratuita de Mix Shop Digital. Encontrá más herramientas gratuitas y programas para tu vida diaria y tu negocio en nuestro sitio.</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="B30" s="76" t="inlineStr">
+      <c r="B30" s="82" t="inlineStr">
         <is>
           <t>→ mixshopdigital.com.py</t>
         </is>
       </c>
     </row>
     <row r="32" ht="8" customHeight="1">
-      <c r="B32" s="43" t="n"/>
+      <c r="B32" s="49" t="n"/>
     </row>
     <row r="33" ht="16" customHeight="1">
-      <c r="B33" s="44" t="inlineStr">
+      <c r="B33" s="50" t="inlineStr">
         <is>
           <t>MIX SHOP DIGITAL  ·  Herramientas inteligentes que simplifican tu vida.</t>
         </is>
       </c>
     </row>
     <row r="34" ht="16" customHeight="1">
-      <c r="B34" s="45" t="inlineStr">
+      <c r="B34" s="51" t="inlineStr">
         <is>
           <t>Versión gratuita  ·  Más herramientas gratuitas para tu vida diaria  →  mixshopdigital.com.py</t>
         </is>
@@ -4190,7 +4431,7 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="1" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="1" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="ECF5"/>
-  <mergeCells count="29">
+  <mergeCells count="28">
     <mergeCell ref="B9:H9"/>
     <mergeCell ref="D1:H1"/>
     <mergeCell ref="B6:H6"/>
@@ -4205,7 +4446,6 @@
     <mergeCell ref="B7:H7"/>
     <mergeCell ref="B25:H25"/>
     <mergeCell ref="B1:C1"/>
-    <mergeCell ref="B3:H3"/>
     <mergeCell ref="B22:H22"/>
     <mergeCell ref="B18:H18"/>
     <mergeCell ref="B21:H21"/>
@@ -4237,5 +4477,6 @@
     <firstHeader/>
     <firstFooter/>
   </headerFooter>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>